<commit_message>
feat: improve carton procurement and customer library
</commit_message>
<xml_diff>
--- a/public/templates/carton-history-order-import-template.xlsx
+++ b/public/templates/carton-history-order-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="历史订单导入" sheetId="1" r:id="R2d9ede09a9254181"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="2" r:id="Ra1aad53cc63c4552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R6160a99718204bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="历史订单导入" sheetId="1" r:id="R17e9b8e0179f4657"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="2" r:id="Rb5b8215c4f2d41c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R7d0e2dd947724d52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,12 +15,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="#,##0.######"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="202" formatCode="0.########"/>
     <x:numFmt numFmtId="203" formatCode="#,##0.000000"/>
     <x:numFmt numFmtId="204" formatCode="#,##0.####"/>
+    <x:numFmt numFmtId="205" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -209,7 +210,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="100">
+  <x:cellXfs count="105">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -447,6 +448,21 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -728,7 +744,7 @@
         <x:v>规格单位</x:v>
       </x:c>
       <x:c r="N5" s="22" t="str">
-        <x:v>单件用量*</x:v>
+        <x:v>每箱个数*</x:v>
       </x:c>
       <x:c r="O5" s="22" t="str">
         <x:v>纸品单位*</x:v>
@@ -746,7 +762,7 @@
         <x:v>明细备注</x:v>
       </x:c>
       <x:c r="T5" s="23" t="str">
-        <x:v>需求数量（自动校验）</x:v>
+        <x:v>纸箱数量（自动校验）</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -769,8 +785,8 @@
       <x:c r="Q6" s="35"/>
       <x:c r="R6" s="35"/>
       <x:c r="S6" s="35"/>
-      <x:c r="T6" s="58" t="str">
-        <x:f>IF(OR(F6="",N6=""),"",F6*N6)</x:f>
+      <x:c r="T6" s="100" t="str">
+        <x:f>IF(OR(F6="",N6="",N6&lt;=0),"",ROUNDUP(F6/N6,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -793,8 +809,8 @@
       <x:c r="Q7" s="38"/>
       <x:c r="R7" s="38"/>
       <x:c r="S7" s="38"/>
-      <x:c r="T7" s="59" t="str">
-        <x:f>IF(OR(F7="",N7=""),"",F7*N7)</x:f>
+      <x:c r="T7" s="101" t="str">
+        <x:f>IF(OR(F7="",N7="",N7&lt;=0),"",ROUNDUP(F7/N7,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -817,8 +833,8 @@
       <x:c r="Q8" s="38"/>
       <x:c r="R8" s="38"/>
       <x:c r="S8" s="38"/>
-      <x:c r="T8" s="59" t="str">
-        <x:f>IF(OR(F8="",N8=""),"",F8*N8)</x:f>
+      <x:c r="T8" s="101" t="str">
+        <x:f>IF(OR(F8="",N8="",N8&lt;=0),"",ROUNDUP(F8/N8,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -841,8 +857,8 @@
       <x:c r="Q9" s="38"/>
       <x:c r="R9" s="38"/>
       <x:c r="S9" s="38"/>
-      <x:c r="T9" s="59" t="str">
-        <x:f>IF(OR(F9="",N9=""),"",F9*N9)</x:f>
+      <x:c r="T9" s="101" t="str">
+        <x:f>IF(OR(F9="",N9="",N9&lt;=0),"",ROUNDUP(F9/N9,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -865,8 +881,8 @@
       <x:c r="Q10" s="38"/>
       <x:c r="R10" s="38"/>
       <x:c r="S10" s="38"/>
-      <x:c r="T10" s="59" t="str">
-        <x:f>IF(OR(F10="",N10=""),"",F10*N10)</x:f>
+      <x:c r="T10" s="101" t="str">
+        <x:f>IF(OR(F10="",N10="",N10&lt;=0),"",ROUNDUP(F10/N10,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -889,8 +905,8 @@
       <x:c r="Q11" s="38"/>
       <x:c r="R11" s="38"/>
       <x:c r="S11" s="38"/>
-      <x:c r="T11" s="59" t="str">
-        <x:f>IF(OR(F11="",N11=""),"",F11*N11)</x:f>
+      <x:c r="T11" s="101" t="str">
+        <x:f>IF(OR(F11="",N11="",N11&lt;=0),"",ROUNDUP(F11/N11,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -913,8 +929,8 @@
       <x:c r="Q12" s="38"/>
       <x:c r="R12" s="38"/>
       <x:c r="S12" s="38"/>
-      <x:c r="T12" s="59" t="str">
-        <x:f>IF(OR(F12="",N12=""),"",F12*N12)</x:f>
+      <x:c r="T12" s="101" t="str">
+        <x:f>IF(OR(F12="",N12="",N12&lt;=0),"",ROUNDUP(F12/N12,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -937,8 +953,8 @@
       <x:c r="Q13" s="38"/>
       <x:c r="R13" s="38"/>
       <x:c r="S13" s="38"/>
-      <x:c r="T13" s="59" t="str">
-        <x:f>IF(OR(F13="",N13=""),"",F13*N13)</x:f>
+      <x:c r="T13" s="101" t="str">
+        <x:f>IF(OR(F13="",N13="",N13&lt;=0),"",ROUNDUP(F13/N13,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -961,8 +977,8 @@
       <x:c r="Q14" s="38"/>
       <x:c r="R14" s="38"/>
       <x:c r="S14" s="38"/>
-      <x:c r="T14" s="59" t="str">
-        <x:f>IF(OR(F14="",N14=""),"",F14*N14)</x:f>
+      <x:c r="T14" s="101" t="str">
+        <x:f>IF(OR(F14="",N14="",N14&lt;=0),"",ROUNDUP(F14/N14,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -985,8 +1001,8 @@
       <x:c r="Q15" s="38"/>
       <x:c r="R15" s="38"/>
       <x:c r="S15" s="38"/>
-      <x:c r="T15" s="59" t="str">
-        <x:f>IF(OR(F15="",N15=""),"",F15*N15)</x:f>
+      <x:c r="T15" s="101" t="str">
+        <x:f>IF(OR(F15="",N15="",N15&lt;=0),"",ROUNDUP(F15/N15,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1009,8 +1025,8 @@
       <x:c r="Q16" s="38"/>
       <x:c r="R16" s="38"/>
       <x:c r="S16" s="38"/>
-      <x:c r="T16" s="59" t="str">
-        <x:f>IF(OR(F16="",N16=""),"",F16*N16)</x:f>
+      <x:c r="T16" s="101" t="str">
+        <x:f>IF(OR(F16="",N16="",N16&lt;=0),"",ROUNDUP(F16/N16,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1033,8 +1049,8 @@
       <x:c r="Q17" s="38"/>
       <x:c r="R17" s="38"/>
       <x:c r="S17" s="38"/>
-      <x:c r="T17" s="59" t="str">
-        <x:f>IF(OR(F17="",N17=""),"",F17*N17)</x:f>
+      <x:c r="T17" s="101" t="str">
+        <x:f>IF(OR(F17="",N17="",N17&lt;=0),"",ROUNDUP(F17/N17,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1057,8 +1073,8 @@
       <x:c r="Q18" s="38"/>
       <x:c r="R18" s="38"/>
       <x:c r="S18" s="38"/>
-      <x:c r="T18" s="59" t="str">
-        <x:f>IF(OR(F18="",N18=""),"",F18*N18)</x:f>
+      <x:c r="T18" s="101" t="str">
+        <x:f>IF(OR(F18="",N18="",N18&lt;=0),"",ROUNDUP(F18/N18,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1081,8 +1097,8 @@
       <x:c r="Q19" s="38"/>
       <x:c r="R19" s="38"/>
       <x:c r="S19" s="38"/>
-      <x:c r="T19" s="59" t="str">
-        <x:f>IF(OR(F19="",N19=""),"",F19*N19)</x:f>
+      <x:c r="T19" s="101" t="str">
+        <x:f>IF(OR(F19="",N19="",N19&lt;=0),"",ROUNDUP(F19/N19,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1105,8 +1121,8 @@
       <x:c r="Q20" s="38"/>
       <x:c r="R20" s="38"/>
       <x:c r="S20" s="38"/>
-      <x:c r="T20" s="59" t="str">
-        <x:f>IF(OR(F20="",N20=""),"",F20*N20)</x:f>
+      <x:c r="T20" s="101" t="str">
+        <x:f>IF(OR(F20="",N20="",N20&lt;=0),"",ROUNDUP(F20/N20,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1129,8 +1145,8 @@
       <x:c r="Q21" s="38"/>
       <x:c r="R21" s="38"/>
       <x:c r="S21" s="38"/>
-      <x:c r="T21" s="59" t="str">
-        <x:f>IF(OR(F21="",N21=""),"",F21*N21)</x:f>
+      <x:c r="T21" s="101" t="str">
+        <x:f>IF(OR(F21="",N21="",N21&lt;=0),"",ROUNDUP(F21/N21,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1153,8 +1169,8 @@
       <x:c r="Q22" s="38"/>
       <x:c r="R22" s="38"/>
       <x:c r="S22" s="38"/>
-      <x:c r="T22" s="59" t="str">
-        <x:f>IF(OR(F22="",N22=""),"",F22*N22)</x:f>
+      <x:c r="T22" s="101" t="str">
+        <x:f>IF(OR(F22="",N22="",N22&lt;=0),"",ROUNDUP(F22/N22,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1177,8 +1193,8 @@
       <x:c r="Q23" s="38"/>
       <x:c r="R23" s="38"/>
       <x:c r="S23" s="38"/>
-      <x:c r="T23" s="59" t="str">
-        <x:f>IF(OR(F23="",N23=""),"",F23*N23)</x:f>
+      <x:c r="T23" s="101" t="str">
+        <x:f>IF(OR(F23="",N23="",N23&lt;=0),"",ROUNDUP(F23/N23,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1201,8 +1217,8 @@
       <x:c r="Q24" s="38"/>
       <x:c r="R24" s="38"/>
       <x:c r="S24" s="38"/>
-      <x:c r="T24" s="59" t="str">
-        <x:f>IF(OR(F24="",N24=""),"",F24*N24)</x:f>
+      <x:c r="T24" s="101" t="str">
+        <x:f>IF(OR(F24="",N24="",N24&lt;=0),"",ROUNDUP(F24/N24,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1225,8 +1241,8 @@
       <x:c r="Q25" s="38"/>
       <x:c r="R25" s="38"/>
       <x:c r="S25" s="38"/>
-      <x:c r="T25" s="59" t="str">
-        <x:f>IF(OR(F25="",N25=""),"",F25*N25)</x:f>
+      <x:c r="T25" s="101" t="str">
+        <x:f>IF(OR(F25="",N25="",N25&lt;=0),"",ROUNDUP(F25/N25,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1249,8 +1265,8 @@
       <x:c r="Q26" s="38"/>
       <x:c r="R26" s="38"/>
       <x:c r="S26" s="38"/>
-      <x:c r="T26" s="59" t="str">
-        <x:f>IF(OR(F26="",N26=""),"",F26*N26)</x:f>
+      <x:c r="T26" s="101" t="str">
+        <x:f>IF(OR(F26="",N26="",N26&lt;=0),"",ROUNDUP(F26/N26,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1273,8 +1289,8 @@
       <x:c r="Q27" s="38"/>
       <x:c r="R27" s="38"/>
       <x:c r="S27" s="38"/>
-      <x:c r="T27" s="59" t="str">
-        <x:f>IF(OR(F27="",N27=""),"",F27*N27)</x:f>
+      <x:c r="T27" s="101" t="str">
+        <x:f>IF(OR(F27="",N27="",N27&lt;=0),"",ROUNDUP(F27/N27,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1297,8 +1313,8 @@
       <x:c r="Q28" s="38"/>
       <x:c r="R28" s="38"/>
       <x:c r="S28" s="38"/>
-      <x:c r="T28" s="59" t="str">
-        <x:f>IF(OR(F28="",N28=""),"",F28*N28)</x:f>
+      <x:c r="T28" s="101" t="str">
+        <x:f>IF(OR(F28="",N28="",N28&lt;=0),"",ROUNDUP(F28/N28,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1321,8 +1337,8 @@
       <x:c r="Q29" s="38"/>
       <x:c r="R29" s="38"/>
       <x:c r="S29" s="38"/>
-      <x:c r="T29" s="59" t="str">
-        <x:f>IF(OR(F29="",N29=""),"",F29*N29)</x:f>
+      <x:c r="T29" s="101" t="str">
+        <x:f>IF(OR(F29="",N29="",N29&lt;=0),"",ROUNDUP(F29/N29,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1345,8 +1361,8 @@
       <x:c r="Q30" s="38"/>
       <x:c r="R30" s="38"/>
       <x:c r="S30" s="38"/>
-      <x:c r="T30" s="59" t="str">
-        <x:f>IF(OR(F30="",N30=""),"",F30*N30)</x:f>
+      <x:c r="T30" s="101" t="str">
+        <x:f>IF(OR(F30="",N30="",N30&lt;=0),"",ROUNDUP(F30/N30,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1369,8 +1385,8 @@
       <x:c r="Q31" s="38"/>
       <x:c r="R31" s="38"/>
       <x:c r="S31" s="38"/>
-      <x:c r="T31" s="59" t="str">
-        <x:f>IF(OR(F31="",N31=""),"",F31*N31)</x:f>
+      <x:c r="T31" s="101" t="str">
+        <x:f>IF(OR(F31="",N31="",N31&lt;=0),"",ROUNDUP(F31/N31,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -1393,8 +1409,8 @@
       <x:c r="Q32" s="38"/>
       <x:c r="R32" s="38"/>
       <x:c r="S32" s="38"/>
-      <x:c r="T32" s="59" t="str">
-        <x:f>IF(OR(F32="",N32=""),"",F32*N32)</x:f>
+      <x:c r="T32" s="101" t="str">
+        <x:f>IF(OR(F32="",N32="",N32&lt;=0),"",ROUNDUP(F32/N32,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -1417,8 +1433,8 @@
       <x:c r="Q33" s="38"/>
       <x:c r="R33" s="38"/>
       <x:c r="S33" s="38"/>
-      <x:c r="T33" s="59" t="str">
-        <x:f>IF(OR(F33="",N33=""),"",F33*N33)</x:f>
+      <x:c r="T33" s="101" t="str">
+        <x:f>IF(OR(F33="",N33="",N33&lt;=0),"",ROUNDUP(F33/N33,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -1441,8 +1457,8 @@
       <x:c r="Q34" s="38"/>
       <x:c r="R34" s="38"/>
       <x:c r="S34" s="38"/>
-      <x:c r="T34" s="59" t="str">
-        <x:f>IF(OR(F34="",N34=""),"",F34*N34)</x:f>
+      <x:c r="T34" s="101" t="str">
+        <x:f>IF(OR(F34="",N34="",N34&lt;=0),"",ROUNDUP(F34/N34,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1465,8 +1481,8 @@
       <x:c r="Q35" s="38"/>
       <x:c r="R35" s="38"/>
       <x:c r="S35" s="38"/>
-      <x:c r="T35" s="59" t="str">
-        <x:f>IF(OR(F35="",N35=""),"",F35*N35)</x:f>
+      <x:c r="T35" s="101" t="str">
+        <x:f>IF(OR(F35="",N35="",N35&lt;=0),"",ROUNDUP(F35/N35,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1489,8 +1505,8 @@
       <x:c r="Q36" s="38"/>
       <x:c r="R36" s="38"/>
       <x:c r="S36" s="38"/>
-      <x:c r="T36" s="59" t="str">
-        <x:f>IF(OR(F36="",N36=""),"",F36*N36)</x:f>
+      <x:c r="T36" s="101" t="str">
+        <x:f>IF(OR(F36="",N36="",N36&lt;=0),"",ROUNDUP(F36/N36,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1513,8 +1529,8 @@
       <x:c r="Q37" s="38"/>
       <x:c r="R37" s="38"/>
       <x:c r="S37" s="38"/>
-      <x:c r="T37" s="59" t="str">
-        <x:f>IF(OR(F37="",N37=""),"",F37*N37)</x:f>
+      <x:c r="T37" s="101" t="str">
+        <x:f>IF(OR(F37="",N37="",N37&lt;=0),"",ROUNDUP(F37/N37,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1537,8 +1553,8 @@
       <x:c r="Q38" s="38"/>
       <x:c r="R38" s="38"/>
       <x:c r="S38" s="38"/>
-      <x:c r="T38" s="59" t="str">
-        <x:f>IF(OR(F38="",N38=""),"",F38*N38)</x:f>
+      <x:c r="T38" s="101" t="str">
+        <x:f>IF(OR(F38="",N38="",N38&lt;=0),"",ROUNDUP(F38/N38,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -1561,8 +1577,8 @@
       <x:c r="Q39" s="38"/>
       <x:c r="R39" s="38"/>
       <x:c r="S39" s="38"/>
-      <x:c r="T39" s="59" t="str">
-        <x:f>IF(OR(F39="",N39=""),"",F39*N39)</x:f>
+      <x:c r="T39" s="101" t="str">
+        <x:f>IF(OR(F39="",N39="",N39&lt;=0),"",ROUNDUP(F39/N39,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -1585,8 +1601,8 @@
       <x:c r="Q40" s="38"/>
       <x:c r="R40" s="38"/>
       <x:c r="S40" s="38"/>
-      <x:c r="T40" s="59" t="str">
-        <x:f>IF(OR(F40="",N40=""),"",F40*N40)</x:f>
+      <x:c r="T40" s="101" t="str">
+        <x:f>IF(OR(F40="",N40="",N40&lt;=0),"",ROUNDUP(F40/N40,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -1609,8 +1625,8 @@
       <x:c r="Q41" s="38"/>
       <x:c r="R41" s="38"/>
       <x:c r="S41" s="38"/>
-      <x:c r="T41" s="59" t="str">
-        <x:f>IF(OR(F41="",N41=""),"",F41*N41)</x:f>
+      <x:c r="T41" s="101" t="str">
+        <x:f>IF(OR(F41="",N41="",N41&lt;=0),"",ROUNDUP(F41/N41,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1633,8 +1649,8 @@
       <x:c r="Q42" s="38"/>
       <x:c r="R42" s="38"/>
       <x:c r="S42" s="38"/>
-      <x:c r="T42" s="59" t="str">
-        <x:f>IF(OR(F42="",N42=""),"",F42*N42)</x:f>
+      <x:c r="T42" s="101" t="str">
+        <x:f>IF(OR(F42="",N42="",N42&lt;=0),"",ROUNDUP(F42/N42,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -1657,8 +1673,8 @@
       <x:c r="Q43" s="38"/>
       <x:c r="R43" s="38"/>
       <x:c r="S43" s="38"/>
-      <x:c r="T43" s="59" t="str">
-        <x:f>IF(OR(F43="",N43=""),"",F43*N43)</x:f>
+      <x:c r="T43" s="101" t="str">
+        <x:f>IF(OR(F43="",N43="",N43&lt;=0),"",ROUNDUP(F43/N43,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -1681,8 +1697,8 @@
       <x:c r="Q44" s="38"/>
       <x:c r="R44" s="38"/>
       <x:c r="S44" s="38"/>
-      <x:c r="T44" s="59" t="str">
-        <x:f>IF(OR(F44="",N44=""),"",F44*N44)</x:f>
+      <x:c r="T44" s="101" t="str">
+        <x:f>IF(OR(F44="",N44="",N44&lt;=0),"",ROUNDUP(F44/N44,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -1705,8 +1721,8 @@
       <x:c r="Q45" s="38"/>
       <x:c r="R45" s="38"/>
       <x:c r="S45" s="38"/>
-      <x:c r="T45" s="59" t="str">
-        <x:f>IF(OR(F45="",N45=""),"",F45*N45)</x:f>
+      <x:c r="T45" s="101" t="str">
+        <x:f>IF(OR(F45="",N45="",N45&lt;=0),"",ROUNDUP(F45/N45,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -1729,8 +1745,8 @@
       <x:c r="Q46" s="38"/>
       <x:c r="R46" s="38"/>
       <x:c r="S46" s="38"/>
-      <x:c r="T46" s="59" t="str">
-        <x:f>IF(OR(F46="",N46=""),"",F46*N46)</x:f>
+      <x:c r="T46" s="101" t="str">
+        <x:f>IF(OR(F46="",N46="",N46&lt;=0),"",ROUNDUP(F46/N46,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -1753,8 +1769,8 @@
       <x:c r="Q47" s="38"/>
       <x:c r="R47" s="38"/>
       <x:c r="S47" s="38"/>
-      <x:c r="T47" s="59" t="str">
-        <x:f>IF(OR(F47="",N47=""),"",F47*N47)</x:f>
+      <x:c r="T47" s="101" t="str">
+        <x:f>IF(OR(F47="",N47="",N47&lt;=0),"",ROUNDUP(F47/N47,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -1777,8 +1793,8 @@
       <x:c r="Q48" s="38"/>
       <x:c r="R48" s="38"/>
       <x:c r="S48" s="38"/>
-      <x:c r="T48" s="59" t="str">
-        <x:f>IF(OR(F48="",N48=""),"",F48*N48)</x:f>
+      <x:c r="T48" s="101" t="str">
+        <x:f>IF(OR(F48="",N48="",N48&lt;=0),"",ROUNDUP(F48/N48,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -1801,8 +1817,8 @@
       <x:c r="Q49" s="38"/>
       <x:c r="R49" s="38"/>
       <x:c r="S49" s="38"/>
-      <x:c r="T49" s="59" t="str">
-        <x:f>IF(OR(F49="",N49=""),"",F49*N49)</x:f>
+      <x:c r="T49" s="101" t="str">
+        <x:f>IF(OR(F49="",N49="",N49&lt;=0),"",ROUNDUP(F49/N49,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -1825,8 +1841,8 @@
       <x:c r="Q50" s="38"/>
       <x:c r="R50" s="38"/>
       <x:c r="S50" s="38"/>
-      <x:c r="T50" s="59" t="str">
-        <x:f>IF(OR(F50="",N50=""),"",F50*N50)</x:f>
+      <x:c r="T50" s="101" t="str">
+        <x:f>IF(OR(F50="",N50="",N50&lt;=0),"",ROUNDUP(F50/N50,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -1849,8 +1865,8 @@
       <x:c r="Q51" s="38"/>
       <x:c r="R51" s="38"/>
       <x:c r="S51" s="38"/>
-      <x:c r="T51" s="59" t="str">
-        <x:f>IF(OR(F51="",N51=""),"",F51*N51)</x:f>
+      <x:c r="T51" s="101" t="str">
+        <x:f>IF(OR(F51="",N51="",N51&lt;=0),"",ROUNDUP(F51/N51,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -1873,8 +1889,8 @@
       <x:c r="Q52" s="38"/>
       <x:c r="R52" s="38"/>
       <x:c r="S52" s="38"/>
-      <x:c r="T52" s="59" t="str">
-        <x:f>IF(OR(F52="",N52=""),"",F52*N52)</x:f>
+      <x:c r="T52" s="101" t="str">
+        <x:f>IF(OR(F52="",N52="",N52&lt;=0),"",ROUNDUP(F52/N52,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -1897,8 +1913,8 @@
       <x:c r="Q53" s="38"/>
       <x:c r="R53" s="38"/>
       <x:c r="S53" s="38"/>
-      <x:c r="T53" s="59" t="str">
-        <x:f>IF(OR(F53="",N53=""),"",F53*N53)</x:f>
+      <x:c r="T53" s="101" t="str">
+        <x:f>IF(OR(F53="",N53="",N53&lt;=0),"",ROUNDUP(F53/N53,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -1921,8 +1937,8 @@
       <x:c r="Q54" s="38"/>
       <x:c r="R54" s="38"/>
       <x:c r="S54" s="38"/>
-      <x:c r="T54" s="59" t="str">
-        <x:f>IF(OR(F54="",N54=""),"",F54*N54)</x:f>
+      <x:c r="T54" s="101" t="str">
+        <x:f>IF(OR(F54="",N54="",N54&lt;=0),"",ROUNDUP(F54/N54,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -1945,8 +1961,8 @@
       <x:c r="Q55" s="38"/>
       <x:c r="R55" s="38"/>
       <x:c r="S55" s="38"/>
-      <x:c r="T55" s="59" t="str">
-        <x:f>IF(OR(F55="",N55=""),"",F55*N55)</x:f>
+      <x:c r="T55" s="101" t="str">
+        <x:f>IF(OR(F55="",N55="",N55&lt;=0),"",ROUNDUP(F55/N55,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -1969,8 +1985,8 @@
       <x:c r="Q56" s="38"/>
       <x:c r="R56" s="38"/>
       <x:c r="S56" s="38"/>
-      <x:c r="T56" s="59" t="str">
-        <x:f>IF(OR(F56="",N56=""),"",F56*N56)</x:f>
+      <x:c r="T56" s="101" t="str">
+        <x:f>IF(OR(F56="",N56="",N56&lt;=0),"",ROUNDUP(F56/N56,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -1993,8 +2009,8 @@
       <x:c r="Q57" s="38"/>
       <x:c r="R57" s="38"/>
       <x:c r="S57" s="38"/>
-      <x:c r="T57" s="59" t="str">
-        <x:f>IF(OR(F57="",N57=""),"",F57*N57)</x:f>
+      <x:c r="T57" s="101" t="str">
+        <x:f>IF(OR(F57="",N57="",N57&lt;=0),"",ROUNDUP(F57/N57,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -2017,8 +2033,8 @@
       <x:c r="Q58" s="38"/>
       <x:c r="R58" s="38"/>
       <x:c r="S58" s="38"/>
-      <x:c r="T58" s="59" t="str">
-        <x:f>IF(OR(F58="",N58=""),"",F58*N58)</x:f>
+      <x:c r="T58" s="101" t="str">
+        <x:f>IF(OR(F58="",N58="",N58&lt;=0),"",ROUNDUP(F58/N58,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -2041,8 +2057,8 @@
       <x:c r="Q59" s="38"/>
       <x:c r="R59" s="38"/>
       <x:c r="S59" s="38"/>
-      <x:c r="T59" s="59" t="str">
-        <x:f>IF(OR(F59="",N59=""),"",F59*N59)</x:f>
+      <x:c r="T59" s="101" t="str">
+        <x:f>IF(OR(F59="",N59="",N59&lt;=0),"",ROUNDUP(F59/N59,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -2065,8 +2081,8 @@
       <x:c r="Q60" s="38"/>
       <x:c r="R60" s="38"/>
       <x:c r="S60" s="38"/>
-      <x:c r="T60" s="59" t="str">
-        <x:f>IF(OR(F60="",N60=""),"",F60*N60)</x:f>
+      <x:c r="T60" s="101" t="str">
+        <x:f>IF(OR(F60="",N60="",N60&lt;=0),"",ROUNDUP(F60/N60,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -2089,8 +2105,8 @@
       <x:c r="Q61" s="38"/>
       <x:c r="R61" s="38"/>
       <x:c r="S61" s="38"/>
-      <x:c r="T61" s="59" t="str">
-        <x:f>IF(OR(F61="",N61=""),"",F61*N61)</x:f>
+      <x:c r="T61" s="101" t="str">
+        <x:f>IF(OR(F61="",N61="",N61&lt;=0),"",ROUNDUP(F61/N61,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -2113,8 +2129,8 @@
       <x:c r="Q62" s="38"/>
       <x:c r="R62" s="38"/>
       <x:c r="S62" s="38"/>
-      <x:c r="T62" s="59" t="str">
-        <x:f>IF(OR(F62="",N62=""),"",F62*N62)</x:f>
+      <x:c r="T62" s="101" t="str">
+        <x:f>IF(OR(F62="",N62="",N62&lt;=0),"",ROUNDUP(F62/N62,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -2137,8 +2153,8 @@
       <x:c r="Q63" s="38"/>
       <x:c r="R63" s="38"/>
       <x:c r="S63" s="38"/>
-      <x:c r="T63" s="59" t="str">
-        <x:f>IF(OR(F63="",N63=""),"",F63*N63)</x:f>
+      <x:c r="T63" s="101" t="str">
+        <x:f>IF(OR(F63="",N63="",N63&lt;=0),"",ROUNDUP(F63/N63,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -2161,8 +2177,8 @@
       <x:c r="Q64" s="38"/>
       <x:c r="R64" s="38"/>
       <x:c r="S64" s="38"/>
-      <x:c r="T64" s="59" t="str">
-        <x:f>IF(OR(F64="",N64=""),"",F64*N64)</x:f>
+      <x:c r="T64" s="101" t="str">
+        <x:f>IF(OR(F64="",N64="",N64&lt;=0),"",ROUNDUP(F64/N64,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -2185,8 +2201,8 @@
       <x:c r="Q65" s="38"/>
       <x:c r="R65" s="38"/>
       <x:c r="S65" s="38"/>
-      <x:c r="T65" s="59" t="str">
-        <x:f>IF(OR(F65="",N65=""),"",F65*N65)</x:f>
+      <x:c r="T65" s="101" t="str">
+        <x:f>IF(OR(F65="",N65="",N65&lt;=0),"",ROUNDUP(F65/N65,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -2209,8 +2225,8 @@
       <x:c r="Q66" s="38"/>
       <x:c r="R66" s="38"/>
       <x:c r="S66" s="38"/>
-      <x:c r="T66" s="59" t="str">
-        <x:f>IF(OR(F66="",N66=""),"",F66*N66)</x:f>
+      <x:c r="T66" s="101" t="str">
+        <x:f>IF(OR(F66="",N66="",N66&lt;=0),"",ROUNDUP(F66/N66,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -2233,8 +2249,8 @@
       <x:c r="Q67" s="38"/>
       <x:c r="R67" s="38"/>
       <x:c r="S67" s="38"/>
-      <x:c r="T67" s="59" t="str">
-        <x:f>IF(OR(F67="",N67=""),"",F67*N67)</x:f>
+      <x:c r="T67" s="101" t="str">
+        <x:f>IF(OR(F67="",N67="",N67&lt;=0),"",ROUNDUP(F67/N67,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -2257,8 +2273,8 @@
       <x:c r="Q68" s="38"/>
       <x:c r="R68" s="38"/>
       <x:c r="S68" s="38"/>
-      <x:c r="T68" s="59" t="str">
-        <x:f>IF(OR(F68="",N68=""),"",F68*N68)</x:f>
+      <x:c r="T68" s="101" t="str">
+        <x:f>IF(OR(F68="",N68="",N68&lt;=0),"",ROUNDUP(F68/N68,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -2281,8 +2297,8 @@
       <x:c r="Q69" s="38"/>
       <x:c r="R69" s="38"/>
       <x:c r="S69" s="38"/>
-      <x:c r="T69" s="59" t="str">
-        <x:f>IF(OR(F69="",N69=""),"",F69*N69)</x:f>
+      <x:c r="T69" s="101" t="str">
+        <x:f>IF(OR(F69="",N69="",N69&lt;=0),"",ROUNDUP(F69/N69,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -2305,8 +2321,8 @@
       <x:c r="Q70" s="38"/>
       <x:c r="R70" s="38"/>
       <x:c r="S70" s="38"/>
-      <x:c r="T70" s="59" t="str">
-        <x:f>IF(OR(F70="",N70=""),"",F70*N70)</x:f>
+      <x:c r="T70" s="101" t="str">
+        <x:f>IF(OR(F70="",N70="",N70&lt;=0),"",ROUNDUP(F70/N70,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -2329,8 +2345,8 @@
       <x:c r="Q71" s="38"/>
       <x:c r="R71" s="38"/>
       <x:c r="S71" s="38"/>
-      <x:c r="T71" s="59" t="str">
-        <x:f>IF(OR(F71="",N71=""),"",F71*N71)</x:f>
+      <x:c r="T71" s="101" t="str">
+        <x:f>IF(OR(F71="",N71="",N71&lt;=0),"",ROUNDUP(F71/N71,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -2353,8 +2369,8 @@
       <x:c r="Q72" s="38"/>
       <x:c r="R72" s="38"/>
       <x:c r="S72" s="38"/>
-      <x:c r="T72" s="59" t="str">
-        <x:f>IF(OR(F72="",N72=""),"",F72*N72)</x:f>
+      <x:c r="T72" s="101" t="str">
+        <x:f>IF(OR(F72="",N72="",N72&lt;=0),"",ROUNDUP(F72/N72,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -2377,8 +2393,8 @@
       <x:c r="Q73" s="38"/>
       <x:c r="R73" s="38"/>
       <x:c r="S73" s="38"/>
-      <x:c r="T73" s="59" t="str">
-        <x:f>IF(OR(F73="",N73=""),"",F73*N73)</x:f>
+      <x:c r="T73" s="101" t="str">
+        <x:f>IF(OR(F73="",N73="",N73&lt;=0),"",ROUNDUP(F73/N73,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -2401,8 +2417,8 @@
       <x:c r="Q74" s="38"/>
       <x:c r="R74" s="38"/>
       <x:c r="S74" s="38"/>
-      <x:c r="T74" s="59" t="str">
-        <x:f>IF(OR(F74="",N74=""),"",F74*N74)</x:f>
+      <x:c r="T74" s="101" t="str">
+        <x:f>IF(OR(F74="",N74="",N74&lt;=0),"",ROUNDUP(F74/N74,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -2425,8 +2441,8 @@
       <x:c r="Q75" s="38"/>
       <x:c r="R75" s="38"/>
       <x:c r="S75" s="38"/>
-      <x:c r="T75" s="59" t="str">
-        <x:f>IF(OR(F75="",N75=""),"",F75*N75)</x:f>
+      <x:c r="T75" s="101" t="str">
+        <x:f>IF(OR(F75="",N75="",N75&lt;=0),"",ROUNDUP(F75/N75,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -2449,8 +2465,8 @@
       <x:c r="Q76" s="38"/>
       <x:c r="R76" s="38"/>
       <x:c r="S76" s="38"/>
-      <x:c r="T76" s="59" t="str">
-        <x:f>IF(OR(F76="",N76=""),"",F76*N76)</x:f>
+      <x:c r="T76" s="101" t="str">
+        <x:f>IF(OR(F76="",N76="",N76&lt;=0),"",ROUNDUP(F76/N76,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -2473,8 +2489,8 @@
       <x:c r="Q77" s="38"/>
       <x:c r="R77" s="38"/>
       <x:c r="S77" s="38"/>
-      <x:c r="T77" s="59" t="str">
-        <x:f>IF(OR(F77="",N77=""),"",F77*N77)</x:f>
+      <x:c r="T77" s="101" t="str">
+        <x:f>IF(OR(F77="",N77="",N77&lt;=0),"",ROUNDUP(F77/N77,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -2497,8 +2513,8 @@
       <x:c r="Q78" s="38"/>
       <x:c r="R78" s="38"/>
       <x:c r="S78" s="38"/>
-      <x:c r="T78" s="59" t="str">
-        <x:f>IF(OR(F78="",N78=""),"",F78*N78)</x:f>
+      <x:c r="T78" s="101" t="str">
+        <x:f>IF(OR(F78="",N78="",N78&lt;=0),"",ROUNDUP(F78/N78,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -2521,8 +2537,8 @@
       <x:c r="Q79" s="38"/>
       <x:c r="R79" s="38"/>
       <x:c r="S79" s="38"/>
-      <x:c r="T79" s="59" t="str">
-        <x:f>IF(OR(F79="",N79=""),"",F79*N79)</x:f>
+      <x:c r="T79" s="101" t="str">
+        <x:f>IF(OR(F79="",N79="",N79&lt;=0),"",ROUNDUP(F79/N79,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -2545,8 +2561,8 @@
       <x:c r="Q80" s="38"/>
       <x:c r="R80" s="38"/>
       <x:c r="S80" s="38"/>
-      <x:c r="T80" s="59" t="str">
-        <x:f>IF(OR(F80="",N80=""),"",F80*N80)</x:f>
+      <x:c r="T80" s="101" t="str">
+        <x:f>IF(OR(F80="",N80="",N80&lt;=0),"",ROUNDUP(F80/N80,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -2569,8 +2585,8 @@
       <x:c r="Q81" s="38"/>
       <x:c r="R81" s="38"/>
       <x:c r="S81" s="38"/>
-      <x:c r="T81" s="59" t="str">
-        <x:f>IF(OR(F81="",N81=""),"",F81*N81)</x:f>
+      <x:c r="T81" s="101" t="str">
+        <x:f>IF(OR(F81="",N81="",N81&lt;=0),"",ROUNDUP(F81/N81,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -2593,8 +2609,8 @@
       <x:c r="Q82" s="38"/>
       <x:c r="R82" s="38"/>
       <x:c r="S82" s="38"/>
-      <x:c r="T82" s="59" t="str">
-        <x:f>IF(OR(F82="",N82=""),"",F82*N82)</x:f>
+      <x:c r="T82" s="101" t="str">
+        <x:f>IF(OR(F82="",N82="",N82&lt;=0),"",ROUNDUP(F82/N82,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -2617,8 +2633,8 @@
       <x:c r="Q83" s="38"/>
       <x:c r="R83" s="38"/>
       <x:c r="S83" s="38"/>
-      <x:c r="T83" s="59" t="str">
-        <x:f>IF(OR(F83="",N83=""),"",F83*N83)</x:f>
+      <x:c r="T83" s="101" t="str">
+        <x:f>IF(OR(F83="",N83="",N83&lt;=0),"",ROUNDUP(F83/N83,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -2641,8 +2657,8 @@
       <x:c r="Q84" s="38"/>
       <x:c r="R84" s="38"/>
       <x:c r="S84" s="38"/>
-      <x:c r="T84" s="59" t="str">
-        <x:f>IF(OR(F84="",N84=""),"",F84*N84)</x:f>
+      <x:c r="T84" s="101" t="str">
+        <x:f>IF(OR(F84="",N84="",N84&lt;=0),"",ROUNDUP(F84/N84,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -2665,8 +2681,8 @@
       <x:c r="Q85" s="38"/>
       <x:c r="R85" s="38"/>
       <x:c r="S85" s="38"/>
-      <x:c r="T85" s="59" t="str">
-        <x:f>IF(OR(F85="",N85=""),"",F85*N85)</x:f>
+      <x:c r="T85" s="101" t="str">
+        <x:f>IF(OR(F85="",N85="",N85&lt;=0),"",ROUNDUP(F85/N85,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -2689,8 +2705,8 @@
       <x:c r="Q86" s="38"/>
       <x:c r="R86" s="38"/>
       <x:c r="S86" s="38"/>
-      <x:c r="T86" s="59" t="str">
-        <x:f>IF(OR(F86="",N86=""),"",F86*N86)</x:f>
+      <x:c r="T86" s="101" t="str">
+        <x:f>IF(OR(F86="",N86="",N86&lt;=0),"",ROUNDUP(F86/N86,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -2713,8 +2729,8 @@
       <x:c r="Q87" s="38"/>
       <x:c r="R87" s="38"/>
       <x:c r="S87" s="38"/>
-      <x:c r="T87" s="59" t="str">
-        <x:f>IF(OR(F87="",N87=""),"",F87*N87)</x:f>
+      <x:c r="T87" s="101" t="str">
+        <x:f>IF(OR(F87="",N87="",N87&lt;=0),"",ROUNDUP(F87/N87,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -2737,8 +2753,8 @@
       <x:c r="Q88" s="38"/>
       <x:c r="R88" s="38"/>
       <x:c r="S88" s="38"/>
-      <x:c r="T88" s="59" t="str">
-        <x:f>IF(OR(F88="",N88=""),"",F88*N88)</x:f>
+      <x:c r="T88" s="101" t="str">
+        <x:f>IF(OR(F88="",N88="",N88&lt;=0),"",ROUNDUP(F88/N88,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -2761,8 +2777,8 @@
       <x:c r="Q89" s="38"/>
       <x:c r="R89" s="38"/>
       <x:c r="S89" s="38"/>
-      <x:c r="T89" s="59" t="str">
-        <x:f>IF(OR(F89="",N89=""),"",F89*N89)</x:f>
+      <x:c r="T89" s="101" t="str">
+        <x:f>IF(OR(F89="",N89="",N89&lt;=0),"",ROUNDUP(F89/N89,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -2785,8 +2801,8 @@
       <x:c r="Q90" s="38"/>
       <x:c r="R90" s="38"/>
       <x:c r="S90" s="38"/>
-      <x:c r="T90" s="59" t="str">
-        <x:f>IF(OR(F90="",N90=""),"",F90*N90)</x:f>
+      <x:c r="T90" s="101" t="str">
+        <x:f>IF(OR(F90="",N90="",N90&lt;=0),"",ROUNDUP(F90/N90,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -2809,8 +2825,8 @@
       <x:c r="Q91" s="38"/>
       <x:c r="R91" s="38"/>
       <x:c r="S91" s="38"/>
-      <x:c r="T91" s="59" t="str">
-        <x:f>IF(OR(F91="",N91=""),"",F91*N91)</x:f>
+      <x:c r="T91" s="101" t="str">
+        <x:f>IF(OR(F91="",N91="",N91&lt;=0),"",ROUNDUP(F91/N91,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -2833,8 +2849,8 @@
       <x:c r="Q92" s="38"/>
       <x:c r="R92" s="38"/>
       <x:c r="S92" s="38"/>
-      <x:c r="T92" s="59" t="str">
-        <x:f>IF(OR(F92="",N92=""),"",F92*N92)</x:f>
+      <x:c r="T92" s="101" t="str">
+        <x:f>IF(OR(F92="",N92="",N92&lt;=0),"",ROUNDUP(F92/N92,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -2857,8 +2873,8 @@
       <x:c r="Q93" s="38"/>
       <x:c r="R93" s="38"/>
       <x:c r="S93" s="38"/>
-      <x:c r="T93" s="59" t="str">
-        <x:f>IF(OR(F93="",N93=""),"",F93*N93)</x:f>
+      <x:c r="T93" s="101" t="str">
+        <x:f>IF(OR(F93="",N93="",N93&lt;=0),"",ROUNDUP(F93/N93,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -2881,8 +2897,8 @@
       <x:c r="Q94" s="38"/>
       <x:c r="R94" s="38"/>
       <x:c r="S94" s="38"/>
-      <x:c r="T94" s="59" t="str">
-        <x:f>IF(OR(F94="",N94=""),"",F94*N94)</x:f>
+      <x:c r="T94" s="101" t="str">
+        <x:f>IF(OR(F94="",N94="",N94&lt;=0),"",ROUNDUP(F94/N94,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -2905,8 +2921,8 @@
       <x:c r="Q95" s="38"/>
       <x:c r="R95" s="38"/>
       <x:c r="S95" s="38"/>
-      <x:c r="T95" s="59" t="str">
-        <x:f>IF(OR(F95="",N95=""),"",F95*N95)</x:f>
+      <x:c r="T95" s="101" t="str">
+        <x:f>IF(OR(F95="",N95="",N95&lt;=0),"",ROUNDUP(F95/N95,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -2929,8 +2945,8 @@
       <x:c r="Q96" s="38"/>
       <x:c r="R96" s="38"/>
       <x:c r="S96" s="38"/>
-      <x:c r="T96" s="59" t="str">
-        <x:f>IF(OR(F96="",N96=""),"",F96*N96)</x:f>
+      <x:c r="T96" s="101" t="str">
+        <x:f>IF(OR(F96="",N96="",N96&lt;=0),"",ROUNDUP(F96/N96,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -2953,8 +2969,8 @@
       <x:c r="Q97" s="38"/>
       <x:c r="R97" s="38"/>
       <x:c r="S97" s="38"/>
-      <x:c r="T97" s="59" t="str">
-        <x:f>IF(OR(F97="",N97=""),"",F97*N97)</x:f>
+      <x:c r="T97" s="101" t="str">
+        <x:f>IF(OR(F97="",N97="",N97&lt;=0),"",ROUNDUP(F97/N97,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -2977,8 +2993,8 @@
       <x:c r="Q98" s="38"/>
       <x:c r="R98" s="38"/>
       <x:c r="S98" s="38"/>
-      <x:c r="T98" s="59" t="str">
-        <x:f>IF(OR(F98="",N98=""),"",F98*N98)</x:f>
+      <x:c r="T98" s="101" t="str">
+        <x:f>IF(OR(F98="",N98="",N98&lt;=0),"",ROUNDUP(F98/N98,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -3001,8 +3017,8 @@
       <x:c r="Q99" s="38"/>
       <x:c r="R99" s="38"/>
       <x:c r="S99" s="38"/>
-      <x:c r="T99" s="59" t="str">
-        <x:f>IF(OR(F99="",N99=""),"",F99*N99)</x:f>
+      <x:c r="T99" s="101" t="str">
+        <x:f>IF(OR(F99="",N99="",N99&lt;=0),"",ROUNDUP(F99/N99,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -3025,8 +3041,8 @@
       <x:c r="Q100" s="38"/>
       <x:c r="R100" s="38"/>
       <x:c r="S100" s="38"/>
-      <x:c r="T100" s="59" t="str">
-        <x:f>IF(OR(F100="",N100=""),"",F100*N100)</x:f>
+      <x:c r="T100" s="101" t="str">
+        <x:f>IF(OR(F100="",N100="",N100&lt;=0),"",ROUNDUP(F100/N100,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -3049,8 +3065,8 @@
       <x:c r="Q101" s="38"/>
       <x:c r="R101" s="38"/>
       <x:c r="S101" s="38"/>
-      <x:c r="T101" s="59" t="str">
-        <x:f>IF(OR(F101="",N101=""),"",F101*N101)</x:f>
+      <x:c r="T101" s="101" t="str">
+        <x:f>IF(OR(F101="",N101="",N101&lt;=0),"",ROUNDUP(F101/N101,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -3073,8 +3089,8 @@
       <x:c r="Q102" s="38"/>
       <x:c r="R102" s="38"/>
       <x:c r="S102" s="38"/>
-      <x:c r="T102" s="59" t="str">
-        <x:f>IF(OR(F102="",N102=""),"",F102*N102)</x:f>
+      <x:c r="T102" s="101" t="str">
+        <x:f>IF(OR(F102="",N102="",N102&lt;=0),"",ROUNDUP(F102/N102,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -3097,8 +3113,8 @@
       <x:c r="Q103" s="38"/>
       <x:c r="R103" s="38"/>
       <x:c r="S103" s="38"/>
-      <x:c r="T103" s="59" t="str">
-        <x:f>IF(OR(F103="",N103=""),"",F103*N103)</x:f>
+      <x:c r="T103" s="101" t="str">
+        <x:f>IF(OR(F103="",N103="",N103&lt;=0),"",ROUNDUP(F103/N103,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -3121,8 +3137,8 @@
       <x:c r="Q104" s="38"/>
       <x:c r="R104" s="38"/>
       <x:c r="S104" s="38"/>
-      <x:c r="T104" s="59" t="str">
-        <x:f>IF(OR(F104="",N104=""),"",F104*N104)</x:f>
+      <x:c r="T104" s="101" t="str">
+        <x:f>IF(OR(F104="",N104="",N104&lt;=0),"",ROUNDUP(F104/N104,0))</x:f>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -3145,8 +3161,8 @@
       <x:c r="Q105" s="41"/>
       <x:c r="R105" s="41"/>
       <x:c r="S105" s="41"/>
-      <x:c r="T105" s="60" t="str">
-        <x:f>IF(OR(F105="",N105=""),"",F105*N105)</x:f>
+      <x:c r="T105" s="102" t="str">
+        <x:f>IF(OR(F105="",N105="",N105&lt;=0),"",ROUNDUP(F105/N105,0))</x:f>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3255,7 +3271,7 @@
         <x:v>规格单位</x:v>
       </x:c>
       <x:c r="N5" s="22" t="str">
-        <x:v>单件用量*</x:v>
+        <x:v>每箱个数*</x:v>
       </x:c>
       <x:c r="O5" s="22" t="str">
         <x:v>纸品单位*</x:v>
@@ -3273,7 +3289,7 @@
         <x:v>明细备注</x:v>
       </x:c>
       <x:c r="T5" s="23" t="str">
-        <x:v>需求数量（自动校验）</x:v>
+        <x:v>纸箱数量（自动校验）</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3316,8 +3332,8 @@
       <x:c r="M6" s="35" t="str">
         <x:v>in</x:v>
       </x:c>
-      <x:c r="N6" s="35" t="n">
-        <x:v>0.008333333333333333</x:v>
+      <x:c r="N6" s="49" t="n">
+        <x:v>120</x:v>
       </x:c>
       <x:c r="O6" s="35" t="str">
         <x:v>个</x:v>
@@ -3334,8 +3350,8 @@
       <x:c r="S6" s="35" t="str">
         <x:v>外箱明细</x:v>
       </x:c>
-      <x:c r="T6" s="58" t="n">
-        <x:f>F6*N6</x:f>
+      <x:c r="T6" s="100" t="n">
+        <x:f>ROUNDUP(F6/N6,0)</x:f>
         <x:v>30</x:v>
       </x:c>
     </x:row>
@@ -3379,8 +3395,8 @@
       <x:c r="M7" s="38" t="str">
         <x:v>in</x:v>
       </x:c>
-      <x:c r="N7" s="38" t="n">
-        <x:v>0.03333333333333333</x:v>
+      <x:c r="N7" s="50" t="n">
+        <x:v>30</x:v>
       </x:c>
       <x:c r="O7" s="38" t="str">
         <x:v>个</x:v>
@@ -3397,8 +3413,8 @@
       <x:c r="S7" s="38" t="str">
         <x:v>内箱明细</x:v>
       </x:c>
-      <x:c r="T7" s="59" t="n">
-        <x:f>F7*N7</x:f>
+      <x:c r="T7" s="101" t="n">
+        <x:f>ROUNDUP(F7/N7,0)</x:f>
         <x:v>120</x:v>
       </x:c>
     </x:row>
@@ -3442,7 +3458,7 @@
       <x:c r="M8" s="38" t="str">
         <x:v>in</x:v>
       </x:c>
-      <x:c r="N8" s="38" t="n">
+      <x:c r="N8" s="50" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O8" s="38" t="str">
@@ -3460,8 +3476,8 @@
       <x:c r="S8" s="38" t="str">
         <x:v>滑板纸明细</x:v>
       </x:c>
-      <x:c r="T8" s="59" t="n">
-        <x:f>F8*N8</x:f>
+      <x:c r="T8" s="101" t="n">
+        <x:f>ROUNDUP(F8/N8,0)</x:f>
         <x:v>3600</x:v>
       </x:c>
     </x:row>
@@ -3505,7 +3521,7 @@
       <x:c r="M9" s="38" t="str">
         <x:v>in</x:v>
       </x:c>
-      <x:c r="N9" s="38" t="n">
+      <x:c r="N9" s="50" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="O9" s="38" t="str">
@@ -3523,8 +3539,8 @@
       <x:c r="S9" s="38" t="str">
         <x:v>卡纸明细</x:v>
       </x:c>
-      <x:c r="T9" s="59" t="n">
-        <x:f>F9*N9</x:f>
+      <x:c r="T9" s="101" t="n">
+        <x:f>ROUNDUP(F9/N9,0)</x:f>
         <x:v>3600</x:v>
       </x:c>
     </x:row>
@@ -3542,13 +3558,15 @@
       <x:c r="K10" s="38"/>
       <x:c r="L10" s="38"/>
       <x:c r="M10" s="38"/>
-      <x:c r="N10" s="38"/>
+      <x:c r="N10" s="50"/>
       <x:c r="O10" s="38"/>
       <x:c r="P10" s="38"/>
       <x:c r="Q10" s="38"/>
       <x:c r="R10" s="38"/>
       <x:c r="S10" s="38"/>
-      <x:c r="T10" s="39"/>
+      <x:c r="T10" s="103" t="str">
+        <x:f>IF(OR(F10="",N10="",N10&lt;=0),"",ROUNDUP(F10/N10,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="37"/>
@@ -3564,13 +3582,15 @@
       <x:c r="K11" s="38"/>
       <x:c r="L11" s="38"/>
       <x:c r="M11" s="38"/>
-      <x:c r="N11" s="38"/>
+      <x:c r="N11" s="50"/>
       <x:c r="O11" s="38"/>
       <x:c r="P11" s="38"/>
       <x:c r="Q11" s="38"/>
       <x:c r="R11" s="38"/>
       <x:c r="S11" s="38"/>
-      <x:c r="T11" s="39"/>
+      <x:c r="T11" s="103" t="str">
+        <x:f>IF(OR(F11="",N11="",N11&lt;=0),"",ROUNDUP(F11/N11,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="37"/>
@@ -3586,13 +3606,15 @@
       <x:c r="K12" s="38"/>
       <x:c r="L12" s="38"/>
       <x:c r="M12" s="38"/>
-      <x:c r="N12" s="38"/>
+      <x:c r="N12" s="50"/>
       <x:c r="O12" s="38"/>
       <x:c r="P12" s="38"/>
       <x:c r="Q12" s="38"/>
       <x:c r="R12" s="38"/>
       <x:c r="S12" s="38"/>
-      <x:c r="T12" s="39"/>
+      <x:c r="T12" s="103" t="str">
+        <x:f>IF(OR(F12="",N12="",N12&lt;=0),"",ROUNDUP(F12/N12,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="37"/>
@@ -3608,13 +3630,15 @@
       <x:c r="K13" s="38"/>
       <x:c r="L13" s="38"/>
       <x:c r="M13" s="38"/>
-      <x:c r="N13" s="38"/>
+      <x:c r="N13" s="50"/>
       <x:c r="O13" s="38"/>
       <x:c r="P13" s="38"/>
       <x:c r="Q13" s="38"/>
       <x:c r="R13" s="38"/>
       <x:c r="S13" s="38"/>
-      <x:c r="T13" s="39"/>
+      <x:c r="T13" s="103" t="str">
+        <x:f>IF(OR(F13="",N13="",N13&lt;=0),"",ROUNDUP(F13/N13,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="37"/>
@@ -3630,13 +3654,15 @@
       <x:c r="K14" s="38"/>
       <x:c r="L14" s="38"/>
       <x:c r="M14" s="38"/>
-      <x:c r="N14" s="38"/>
+      <x:c r="N14" s="50"/>
       <x:c r="O14" s="38"/>
       <x:c r="P14" s="38"/>
       <x:c r="Q14" s="38"/>
       <x:c r="R14" s="38"/>
       <x:c r="S14" s="38"/>
-      <x:c r="T14" s="39"/>
+      <x:c r="T14" s="103" t="str">
+        <x:f>IF(OR(F14="",N14="",N14&lt;=0),"",ROUNDUP(F14/N14,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="37"/>
@@ -3652,13 +3678,15 @@
       <x:c r="K15" s="38"/>
       <x:c r="L15" s="38"/>
       <x:c r="M15" s="38"/>
-      <x:c r="N15" s="38"/>
+      <x:c r="N15" s="50"/>
       <x:c r="O15" s="38"/>
       <x:c r="P15" s="38"/>
       <x:c r="Q15" s="38"/>
       <x:c r="R15" s="38"/>
       <x:c r="S15" s="38"/>
-      <x:c r="T15" s="39"/>
+      <x:c r="T15" s="103" t="str">
+        <x:f>IF(OR(F15="",N15="",N15&lt;=0),"",ROUNDUP(F15/N15,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="37"/>
@@ -3674,13 +3702,15 @@
       <x:c r="K16" s="38"/>
       <x:c r="L16" s="38"/>
       <x:c r="M16" s="38"/>
-      <x:c r="N16" s="38"/>
+      <x:c r="N16" s="50"/>
       <x:c r="O16" s="38"/>
       <x:c r="P16" s="38"/>
       <x:c r="Q16" s="38"/>
       <x:c r="R16" s="38"/>
       <x:c r="S16" s="38"/>
-      <x:c r="T16" s="39"/>
+      <x:c r="T16" s="103" t="str">
+        <x:f>IF(OR(F16="",N16="",N16&lt;=0),"",ROUNDUP(F16/N16,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="37"/>
@@ -3696,13 +3726,15 @@
       <x:c r="K17" s="38"/>
       <x:c r="L17" s="38"/>
       <x:c r="M17" s="38"/>
-      <x:c r="N17" s="38"/>
+      <x:c r="N17" s="50"/>
       <x:c r="O17" s="38"/>
       <x:c r="P17" s="38"/>
       <x:c r="Q17" s="38"/>
       <x:c r="R17" s="38"/>
       <x:c r="S17" s="38"/>
-      <x:c r="T17" s="39"/>
+      <x:c r="T17" s="103" t="str">
+        <x:f>IF(OR(F17="",N17="",N17&lt;=0),"",ROUNDUP(F17/N17,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="37"/>
@@ -3718,13 +3750,15 @@
       <x:c r="K18" s="38"/>
       <x:c r="L18" s="38"/>
       <x:c r="M18" s="38"/>
-      <x:c r="N18" s="38"/>
+      <x:c r="N18" s="50"/>
       <x:c r="O18" s="38"/>
       <x:c r="P18" s="38"/>
       <x:c r="Q18" s="38"/>
       <x:c r="R18" s="38"/>
       <x:c r="S18" s="38"/>
-      <x:c r="T18" s="39"/>
+      <x:c r="T18" s="103" t="str">
+        <x:f>IF(OR(F18="",N18="",N18&lt;=0),"",ROUNDUP(F18/N18,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="37"/>
@@ -3740,13 +3774,15 @@
       <x:c r="K19" s="38"/>
       <x:c r="L19" s="38"/>
       <x:c r="M19" s="38"/>
-      <x:c r="N19" s="38"/>
+      <x:c r="N19" s="50"/>
       <x:c r="O19" s="38"/>
       <x:c r="P19" s="38"/>
       <x:c r="Q19" s="38"/>
       <x:c r="R19" s="38"/>
       <x:c r="S19" s="38"/>
-      <x:c r="T19" s="39"/>
+      <x:c r="T19" s="103" t="str">
+        <x:f>IF(OR(F19="",N19="",N19&lt;=0),"",ROUNDUP(F19/N19,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="37"/>
@@ -3762,13 +3798,15 @@
       <x:c r="K20" s="38"/>
       <x:c r="L20" s="38"/>
       <x:c r="M20" s="38"/>
-      <x:c r="N20" s="38"/>
+      <x:c r="N20" s="50"/>
       <x:c r="O20" s="38"/>
       <x:c r="P20" s="38"/>
       <x:c r="Q20" s="38"/>
       <x:c r="R20" s="38"/>
       <x:c r="S20" s="38"/>
-      <x:c r="T20" s="39"/>
+      <x:c r="T20" s="103" t="str">
+        <x:f>IF(OR(F20="",N20="",N20&lt;=0),"",ROUNDUP(F20/N20,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="37"/>
@@ -3784,13 +3822,15 @@
       <x:c r="K21" s="38"/>
       <x:c r="L21" s="38"/>
       <x:c r="M21" s="38"/>
-      <x:c r="N21" s="38"/>
+      <x:c r="N21" s="50"/>
       <x:c r="O21" s="38"/>
       <x:c r="P21" s="38"/>
       <x:c r="Q21" s="38"/>
       <x:c r="R21" s="38"/>
       <x:c r="S21" s="38"/>
-      <x:c r="T21" s="39"/>
+      <x:c r="T21" s="103" t="str">
+        <x:f>IF(OR(F21="",N21="",N21&lt;=0),"",ROUNDUP(F21/N21,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="37"/>
@@ -3806,13 +3846,15 @@
       <x:c r="K22" s="38"/>
       <x:c r="L22" s="38"/>
       <x:c r="M22" s="38"/>
-      <x:c r="N22" s="38"/>
+      <x:c r="N22" s="50"/>
       <x:c r="O22" s="38"/>
       <x:c r="P22" s="38"/>
       <x:c r="Q22" s="38"/>
       <x:c r="R22" s="38"/>
       <x:c r="S22" s="38"/>
-      <x:c r="T22" s="39"/>
+      <x:c r="T22" s="103" t="str">
+        <x:f>IF(OR(F22="",N22="",N22&lt;=0),"",ROUNDUP(F22/N22,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="37"/>
@@ -3828,13 +3870,15 @@
       <x:c r="K23" s="38"/>
       <x:c r="L23" s="38"/>
       <x:c r="M23" s="38"/>
-      <x:c r="N23" s="38"/>
+      <x:c r="N23" s="50"/>
       <x:c r="O23" s="38"/>
       <x:c r="P23" s="38"/>
       <x:c r="Q23" s="38"/>
       <x:c r="R23" s="38"/>
       <x:c r="S23" s="38"/>
-      <x:c r="T23" s="39"/>
+      <x:c r="T23" s="103" t="str">
+        <x:f>IF(OR(F23="",N23="",N23&lt;=0),"",ROUNDUP(F23/N23,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="37"/>
@@ -3850,13 +3894,15 @@
       <x:c r="K24" s="38"/>
       <x:c r="L24" s="38"/>
       <x:c r="M24" s="38"/>
-      <x:c r="N24" s="38"/>
+      <x:c r="N24" s="50"/>
       <x:c r="O24" s="38"/>
       <x:c r="P24" s="38"/>
       <x:c r="Q24" s="38"/>
       <x:c r="R24" s="38"/>
       <x:c r="S24" s="38"/>
-      <x:c r="T24" s="39"/>
+      <x:c r="T24" s="103" t="str">
+        <x:f>IF(OR(F24="",N24="",N24&lt;=0),"",ROUNDUP(F24/N24,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="37"/>
@@ -3872,13 +3918,15 @@
       <x:c r="K25" s="38"/>
       <x:c r="L25" s="38"/>
       <x:c r="M25" s="38"/>
-      <x:c r="N25" s="38"/>
+      <x:c r="N25" s="50"/>
       <x:c r="O25" s="38"/>
       <x:c r="P25" s="38"/>
       <x:c r="Q25" s="38"/>
       <x:c r="R25" s="38"/>
       <x:c r="S25" s="38"/>
-      <x:c r="T25" s="39"/>
+      <x:c r="T25" s="103" t="str">
+        <x:f>IF(OR(F25="",N25="",N25&lt;=0),"",ROUNDUP(F25/N25,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="37"/>
@@ -3894,13 +3942,15 @@
       <x:c r="K26" s="38"/>
       <x:c r="L26" s="38"/>
       <x:c r="M26" s="38"/>
-      <x:c r="N26" s="38"/>
+      <x:c r="N26" s="50"/>
       <x:c r="O26" s="38"/>
       <x:c r="P26" s="38"/>
       <x:c r="Q26" s="38"/>
       <x:c r="R26" s="38"/>
       <x:c r="S26" s="38"/>
-      <x:c r="T26" s="39"/>
+      <x:c r="T26" s="103" t="str">
+        <x:f>IF(OR(F26="",N26="",N26&lt;=0),"",ROUNDUP(F26/N26,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="37"/>
@@ -3916,13 +3966,15 @@
       <x:c r="K27" s="38"/>
       <x:c r="L27" s="38"/>
       <x:c r="M27" s="38"/>
-      <x:c r="N27" s="38"/>
+      <x:c r="N27" s="50"/>
       <x:c r="O27" s="38"/>
       <x:c r="P27" s="38"/>
       <x:c r="Q27" s="38"/>
       <x:c r="R27" s="38"/>
       <x:c r="S27" s="38"/>
-      <x:c r="T27" s="39"/>
+      <x:c r="T27" s="103" t="str">
+        <x:f>IF(OR(F27="",N27="",N27&lt;=0),"",ROUNDUP(F27/N27,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="37"/>
@@ -3938,13 +3990,15 @@
       <x:c r="K28" s="38"/>
       <x:c r="L28" s="38"/>
       <x:c r="M28" s="38"/>
-      <x:c r="N28" s="38"/>
+      <x:c r="N28" s="50"/>
       <x:c r="O28" s="38"/>
       <x:c r="P28" s="38"/>
       <x:c r="Q28" s="38"/>
       <x:c r="R28" s="38"/>
       <x:c r="S28" s="38"/>
-      <x:c r="T28" s="39"/>
+      <x:c r="T28" s="103" t="str">
+        <x:f>IF(OR(F28="",N28="",N28&lt;=0),"",ROUNDUP(F28/N28,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="37"/>
@@ -3960,13 +4014,15 @@
       <x:c r="K29" s="38"/>
       <x:c r="L29" s="38"/>
       <x:c r="M29" s="38"/>
-      <x:c r="N29" s="38"/>
+      <x:c r="N29" s="50"/>
       <x:c r="O29" s="38"/>
       <x:c r="P29" s="38"/>
       <x:c r="Q29" s="38"/>
       <x:c r="R29" s="38"/>
       <x:c r="S29" s="38"/>
-      <x:c r="T29" s="39"/>
+      <x:c r="T29" s="103" t="str">
+        <x:f>IF(OR(F29="",N29="",N29&lt;=0),"",ROUNDUP(F29/N29,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="37"/>
@@ -3982,13 +4038,15 @@
       <x:c r="K30" s="38"/>
       <x:c r="L30" s="38"/>
       <x:c r="M30" s="38"/>
-      <x:c r="N30" s="38"/>
+      <x:c r="N30" s="50"/>
       <x:c r="O30" s="38"/>
       <x:c r="P30" s="38"/>
       <x:c r="Q30" s="38"/>
       <x:c r="R30" s="38"/>
       <x:c r="S30" s="38"/>
-      <x:c r="T30" s="39"/>
+      <x:c r="T30" s="103" t="str">
+        <x:f>IF(OR(F30="",N30="",N30&lt;=0),"",ROUNDUP(F30/N30,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="37"/>
@@ -4004,13 +4062,15 @@
       <x:c r="K31" s="38"/>
       <x:c r="L31" s="38"/>
       <x:c r="M31" s="38"/>
-      <x:c r="N31" s="38"/>
+      <x:c r="N31" s="50"/>
       <x:c r="O31" s="38"/>
       <x:c r="P31" s="38"/>
       <x:c r="Q31" s="38"/>
       <x:c r="R31" s="38"/>
       <x:c r="S31" s="38"/>
-      <x:c r="T31" s="39"/>
+      <x:c r="T31" s="103" t="str">
+        <x:f>IF(OR(F31="",N31="",N31&lt;=0),"",ROUNDUP(F31/N31,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="37"/>
@@ -4026,13 +4086,15 @@
       <x:c r="K32" s="38"/>
       <x:c r="L32" s="38"/>
       <x:c r="M32" s="38"/>
-      <x:c r="N32" s="38"/>
+      <x:c r="N32" s="50"/>
       <x:c r="O32" s="38"/>
       <x:c r="P32" s="38"/>
       <x:c r="Q32" s="38"/>
       <x:c r="R32" s="38"/>
       <x:c r="S32" s="38"/>
-      <x:c r="T32" s="39"/>
+      <x:c r="T32" s="103" t="str">
+        <x:f>IF(OR(F32="",N32="",N32&lt;=0),"",ROUNDUP(F32/N32,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="37"/>
@@ -4048,13 +4110,15 @@
       <x:c r="K33" s="38"/>
       <x:c r="L33" s="38"/>
       <x:c r="M33" s="38"/>
-      <x:c r="N33" s="38"/>
+      <x:c r="N33" s="50"/>
       <x:c r="O33" s="38"/>
       <x:c r="P33" s="38"/>
       <x:c r="Q33" s="38"/>
       <x:c r="R33" s="38"/>
       <x:c r="S33" s="38"/>
-      <x:c r="T33" s="39"/>
+      <x:c r="T33" s="103" t="str">
+        <x:f>IF(OR(F33="",N33="",N33&lt;=0),"",ROUNDUP(F33/N33,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="37"/>
@@ -4070,13 +4134,15 @@
       <x:c r="K34" s="38"/>
       <x:c r="L34" s="38"/>
       <x:c r="M34" s="38"/>
-      <x:c r="N34" s="38"/>
+      <x:c r="N34" s="50"/>
       <x:c r="O34" s="38"/>
       <x:c r="P34" s="38"/>
       <x:c r="Q34" s="38"/>
       <x:c r="R34" s="38"/>
       <x:c r="S34" s="38"/>
-      <x:c r="T34" s="39"/>
+      <x:c r="T34" s="103" t="str">
+        <x:f>IF(OR(F34="",N34="",N34&lt;=0),"",ROUNDUP(F34/N34,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="37"/>
@@ -4092,13 +4158,15 @@
       <x:c r="K35" s="38"/>
       <x:c r="L35" s="38"/>
       <x:c r="M35" s="38"/>
-      <x:c r="N35" s="38"/>
+      <x:c r="N35" s="50"/>
       <x:c r="O35" s="38"/>
       <x:c r="P35" s="38"/>
       <x:c r="Q35" s="38"/>
       <x:c r="R35" s="38"/>
       <x:c r="S35" s="38"/>
-      <x:c r="T35" s="39"/>
+      <x:c r="T35" s="103" t="str">
+        <x:f>IF(OR(F35="",N35="",N35&lt;=0),"",ROUNDUP(F35/N35,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="37"/>
@@ -4114,13 +4182,15 @@
       <x:c r="K36" s="38"/>
       <x:c r="L36" s="38"/>
       <x:c r="M36" s="38"/>
-      <x:c r="N36" s="38"/>
+      <x:c r="N36" s="50"/>
       <x:c r="O36" s="38"/>
       <x:c r="P36" s="38"/>
       <x:c r="Q36" s="38"/>
       <x:c r="R36" s="38"/>
       <x:c r="S36" s="38"/>
-      <x:c r="T36" s="39"/>
+      <x:c r="T36" s="103" t="str">
+        <x:f>IF(OR(F36="",N36="",N36&lt;=0),"",ROUNDUP(F36/N36,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="37"/>
@@ -4136,13 +4206,15 @@
       <x:c r="K37" s="38"/>
       <x:c r="L37" s="38"/>
       <x:c r="M37" s="38"/>
-      <x:c r="N37" s="38"/>
+      <x:c r="N37" s="50"/>
       <x:c r="O37" s="38"/>
       <x:c r="P37" s="38"/>
       <x:c r="Q37" s="38"/>
       <x:c r="R37" s="38"/>
       <x:c r="S37" s="38"/>
-      <x:c r="T37" s="39"/>
+      <x:c r="T37" s="103" t="str">
+        <x:f>IF(OR(F37="",N37="",N37&lt;=0),"",ROUNDUP(F37/N37,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="37"/>
@@ -4158,13 +4230,15 @@
       <x:c r="K38" s="38"/>
       <x:c r="L38" s="38"/>
       <x:c r="M38" s="38"/>
-      <x:c r="N38" s="38"/>
+      <x:c r="N38" s="50"/>
       <x:c r="O38" s="38"/>
       <x:c r="P38" s="38"/>
       <x:c r="Q38" s="38"/>
       <x:c r="R38" s="38"/>
       <x:c r="S38" s="38"/>
-      <x:c r="T38" s="39"/>
+      <x:c r="T38" s="103" t="str">
+        <x:f>IF(OR(F38="",N38="",N38&lt;=0),"",ROUNDUP(F38/N38,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="37"/>
@@ -4180,13 +4254,15 @@
       <x:c r="K39" s="38"/>
       <x:c r="L39" s="38"/>
       <x:c r="M39" s="38"/>
-      <x:c r="N39" s="38"/>
+      <x:c r="N39" s="50"/>
       <x:c r="O39" s="38"/>
       <x:c r="P39" s="38"/>
       <x:c r="Q39" s="38"/>
       <x:c r="R39" s="38"/>
       <x:c r="S39" s="38"/>
-      <x:c r="T39" s="39"/>
+      <x:c r="T39" s="103" t="str">
+        <x:f>IF(OR(F39="",N39="",N39&lt;=0),"",ROUNDUP(F39/N39,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="37"/>
@@ -4202,13 +4278,15 @@
       <x:c r="K40" s="38"/>
       <x:c r="L40" s="38"/>
       <x:c r="M40" s="38"/>
-      <x:c r="N40" s="38"/>
+      <x:c r="N40" s="50"/>
       <x:c r="O40" s="38"/>
       <x:c r="P40" s="38"/>
       <x:c r="Q40" s="38"/>
       <x:c r="R40" s="38"/>
       <x:c r="S40" s="38"/>
-      <x:c r="T40" s="39"/>
+      <x:c r="T40" s="103" t="str">
+        <x:f>IF(OR(F40="",N40="",N40&lt;=0),"",ROUNDUP(F40/N40,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="37"/>
@@ -4224,13 +4302,15 @@
       <x:c r="K41" s="38"/>
       <x:c r="L41" s="38"/>
       <x:c r="M41" s="38"/>
-      <x:c r="N41" s="38"/>
+      <x:c r="N41" s="50"/>
       <x:c r="O41" s="38"/>
       <x:c r="P41" s="38"/>
       <x:c r="Q41" s="38"/>
       <x:c r="R41" s="38"/>
       <x:c r="S41" s="38"/>
-      <x:c r="T41" s="39"/>
+      <x:c r="T41" s="103" t="str">
+        <x:f>IF(OR(F41="",N41="",N41&lt;=0),"",ROUNDUP(F41/N41,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="37"/>
@@ -4246,13 +4326,15 @@
       <x:c r="K42" s="38"/>
       <x:c r="L42" s="38"/>
       <x:c r="M42" s="38"/>
-      <x:c r="N42" s="38"/>
+      <x:c r="N42" s="50"/>
       <x:c r="O42" s="38"/>
       <x:c r="P42" s="38"/>
       <x:c r="Q42" s="38"/>
       <x:c r="R42" s="38"/>
       <x:c r="S42" s="38"/>
-      <x:c r="T42" s="39"/>
+      <x:c r="T42" s="103" t="str">
+        <x:f>IF(OR(F42="",N42="",N42&lt;=0),"",ROUNDUP(F42/N42,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="37"/>
@@ -4268,13 +4350,15 @@
       <x:c r="K43" s="38"/>
       <x:c r="L43" s="38"/>
       <x:c r="M43" s="38"/>
-      <x:c r="N43" s="38"/>
+      <x:c r="N43" s="50"/>
       <x:c r="O43" s="38"/>
       <x:c r="P43" s="38"/>
       <x:c r="Q43" s="38"/>
       <x:c r="R43" s="38"/>
       <x:c r="S43" s="38"/>
-      <x:c r="T43" s="39"/>
+      <x:c r="T43" s="103" t="str">
+        <x:f>IF(OR(F43="",N43="",N43&lt;=0),"",ROUNDUP(F43/N43,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="37"/>
@@ -4290,13 +4374,15 @@
       <x:c r="K44" s="38"/>
       <x:c r="L44" s="38"/>
       <x:c r="M44" s="38"/>
-      <x:c r="N44" s="38"/>
+      <x:c r="N44" s="50"/>
       <x:c r="O44" s="38"/>
       <x:c r="P44" s="38"/>
       <x:c r="Q44" s="38"/>
       <x:c r="R44" s="38"/>
       <x:c r="S44" s="38"/>
-      <x:c r="T44" s="39"/>
+      <x:c r="T44" s="103" t="str">
+        <x:f>IF(OR(F44="",N44="",N44&lt;=0),"",ROUNDUP(F44/N44,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="37"/>
@@ -4312,13 +4398,15 @@
       <x:c r="K45" s="38"/>
       <x:c r="L45" s="38"/>
       <x:c r="M45" s="38"/>
-      <x:c r="N45" s="38"/>
+      <x:c r="N45" s="50"/>
       <x:c r="O45" s="38"/>
       <x:c r="P45" s="38"/>
       <x:c r="Q45" s="38"/>
       <x:c r="R45" s="38"/>
       <x:c r="S45" s="38"/>
-      <x:c r="T45" s="39"/>
+      <x:c r="T45" s="103" t="str">
+        <x:f>IF(OR(F45="",N45="",N45&lt;=0),"",ROUNDUP(F45/N45,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="37"/>
@@ -4334,13 +4422,15 @@
       <x:c r="K46" s="38"/>
       <x:c r="L46" s="38"/>
       <x:c r="M46" s="38"/>
-      <x:c r="N46" s="38"/>
+      <x:c r="N46" s="50"/>
       <x:c r="O46" s="38"/>
       <x:c r="P46" s="38"/>
       <x:c r="Q46" s="38"/>
       <x:c r="R46" s="38"/>
       <x:c r="S46" s="38"/>
-      <x:c r="T46" s="39"/>
+      <x:c r="T46" s="103" t="str">
+        <x:f>IF(OR(F46="",N46="",N46&lt;=0),"",ROUNDUP(F46/N46,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="37"/>
@@ -4356,13 +4446,15 @@
       <x:c r="K47" s="38"/>
       <x:c r="L47" s="38"/>
       <x:c r="M47" s="38"/>
-      <x:c r="N47" s="38"/>
+      <x:c r="N47" s="50"/>
       <x:c r="O47" s="38"/>
       <x:c r="P47" s="38"/>
       <x:c r="Q47" s="38"/>
       <x:c r="R47" s="38"/>
       <x:c r="S47" s="38"/>
-      <x:c r="T47" s="39"/>
+      <x:c r="T47" s="103" t="str">
+        <x:f>IF(OR(F47="",N47="",N47&lt;=0),"",ROUNDUP(F47/N47,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="37"/>
@@ -4378,13 +4470,15 @@
       <x:c r="K48" s="38"/>
       <x:c r="L48" s="38"/>
       <x:c r="M48" s="38"/>
-      <x:c r="N48" s="38"/>
+      <x:c r="N48" s="50"/>
       <x:c r="O48" s="38"/>
       <x:c r="P48" s="38"/>
       <x:c r="Q48" s="38"/>
       <x:c r="R48" s="38"/>
       <x:c r="S48" s="38"/>
-      <x:c r="T48" s="39"/>
+      <x:c r="T48" s="103" t="str">
+        <x:f>IF(OR(F48="",N48="",N48&lt;=0),"",ROUNDUP(F48/N48,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="37"/>
@@ -4400,13 +4494,15 @@
       <x:c r="K49" s="38"/>
       <x:c r="L49" s="38"/>
       <x:c r="M49" s="38"/>
-      <x:c r="N49" s="38"/>
+      <x:c r="N49" s="50"/>
       <x:c r="O49" s="38"/>
       <x:c r="P49" s="38"/>
       <x:c r="Q49" s="38"/>
       <x:c r="R49" s="38"/>
       <x:c r="S49" s="38"/>
-      <x:c r="T49" s="39"/>
+      <x:c r="T49" s="103" t="str">
+        <x:f>IF(OR(F49="",N49="",N49&lt;=0),"",ROUNDUP(F49/N49,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="37"/>
@@ -4422,13 +4518,15 @@
       <x:c r="K50" s="38"/>
       <x:c r="L50" s="38"/>
       <x:c r="M50" s="38"/>
-      <x:c r="N50" s="38"/>
+      <x:c r="N50" s="50"/>
       <x:c r="O50" s="38"/>
       <x:c r="P50" s="38"/>
       <x:c r="Q50" s="38"/>
       <x:c r="R50" s="38"/>
       <x:c r="S50" s="38"/>
-      <x:c r="T50" s="39"/>
+      <x:c r="T50" s="103" t="str">
+        <x:f>IF(OR(F50="",N50="",N50&lt;=0),"",ROUNDUP(F50/N50,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="37"/>
@@ -4444,13 +4542,15 @@
       <x:c r="K51" s="38"/>
       <x:c r="L51" s="38"/>
       <x:c r="M51" s="38"/>
-      <x:c r="N51" s="38"/>
+      <x:c r="N51" s="50"/>
       <x:c r="O51" s="38"/>
       <x:c r="P51" s="38"/>
       <x:c r="Q51" s="38"/>
       <x:c r="R51" s="38"/>
       <x:c r="S51" s="38"/>
-      <x:c r="T51" s="39"/>
+      <x:c r="T51" s="103" t="str">
+        <x:f>IF(OR(F51="",N51="",N51&lt;=0),"",ROUNDUP(F51/N51,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="37"/>
@@ -4466,13 +4566,15 @@
       <x:c r="K52" s="38"/>
       <x:c r="L52" s="38"/>
       <x:c r="M52" s="38"/>
-      <x:c r="N52" s="38"/>
+      <x:c r="N52" s="50"/>
       <x:c r="O52" s="38"/>
       <x:c r="P52" s="38"/>
       <x:c r="Q52" s="38"/>
       <x:c r="R52" s="38"/>
       <x:c r="S52" s="38"/>
-      <x:c r="T52" s="39"/>
+      <x:c r="T52" s="103" t="str">
+        <x:f>IF(OR(F52="",N52="",N52&lt;=0),"",ROUNDUP(F52/N52,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="37"/>
@@ -4488,13 +4590,15 @@
       <x:c r="K53" s="38"/>
       <x:c r="L53" s="38"/>
       <x:c r="M53" s="38"/>
-      <x:c r="N53" s="38"/>
+      <x:c r="N53" s="50"/>
       <x:c r="O53" s="38"/>
       <x:c r="P53" s="38"/>
       <x:c r="Q53" s="38"/>
       <x:c r="R53" s="38"/>
       <x:c r="S53" s="38"/>
-      <x:c r="T53" s="39"/>
+      <x:c r="T53" s="103" t="str">
+        <x:f>IF(OR(F53="",N53="",N53&lt;=0),"",ROUNDUP(F53/N53,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="37"/>
@@ -4510,13 +4614,15 @@
       <x:c r="K54" s="38"/>
       <x:c r="L54" s="38"/>
       <x:c r="M54" s="38"/>
-      <x:c r="N54" s="38"/>
+      <x:c r="N54" s="50"/>
       <x:c r="O54" s="38"/>
       <x:c r="P54" s="38"/>
       <x:c r="Q54" s="38"/>
       <x:c r="R54" s="38"/>
       <x:c r="S54" s="38"/>
-      <x:c r="T54" s="39"/>
+      <x:c r="T54" s="103" t="str">
+        <x:f>IF(OR(F54="",N54="",N54&lt;=0),"",ROUNDUP(F54/N54,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="37"/>
@@ -4532,13 +4638,15 @@
       <x:c r="K55" s="38"/>
       <x:c r="L55" s="38"/>
       <x:c r="M55" s="38"/>
-      <x:c r="N55" s="38"/>
+      <x:c r="N55" s="50"/>
       <x:c r="O55" s="38"/>
       <x:c r="P55" s="38"/>
       <x:c r="Q55" s="38"/>
       <x:c r="R55" s="38"/>
       <x:c r="S55" s="38"/>
-      <x:c r="T55" s="39"/>
+      <x:c r="T55" s="103" t="str">
+        <x:f>IF(OR(F55="",N55="",N55&lt;=0),"",ROUNDUP(F55/N55,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="37"/>
@@ -4554,13 +4662,15 @@
       <x:c r="K56" s="38"/>
       <x:c r="L56" s="38"/>
       <x:c r="M56" s="38"/>
-      <x:c r="N56" s="38"/>
+      <x:c r="N56" s="50"/>
       <x:c r="O56" s="38"/>
       <x:c r="P56" s="38"/>
       <x:c r="Q56" s="38"/>
       <x:c r="R56" s="38"/>
       <x:c r="S56" s="38"/>
-      <x:c r="T56" s="39"/>
+      <x:c r="T56" s="103" t="str">
+        <x:f>IF(OR(F56="",N56="",N56&lt;=0),"",ROUNDUP(F56/N56,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="37"/>
@@ -4576,13 +4686,15 @@
       <x:c r="K57" s="38"/>
       <x:c r="L57" s="38"/>
       <x:c r="M57" s="38"/>
-      <x:c r="N57" s="38"/>
+      <x:c r="N57" s="50"/>
       <x:c r="O57" s="38"/>
       <x:c r="P57" s="38"/>
       <x:c r="Q57" s="38"/>
       <x:c r="R57" s="38"/>
       <x:c r="S57" s="38"/>
-      <x:c r="T57" s="39"/>
+      <x:c r="T57" s="103" t="str">
+        <x:f>IF(OR(F57="",N57="",N57&lt;=0),"",ROUNDUP(F57/N57,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="37"/>
@@ -4598,13 +4710,15 @@
       <x:c r="K58" s="38"/>
       <x:c r="L58" s="38"/>
       <x:c r="M58" s="38"/>
-      <x:c r="N58" s="38"/>
+      <x:c r="N58" s="50"/>
       <x:c r="O58" s="38"/>
       <x:c r="P58" s="38"/>
       <x:c r="Q58" s="38"/>
       <x:c r="R58" s="38"/>
       <x:c r="S58" s="38"/>
-      <x:c r="T58" s="39"/>
+      <x:c r="T58" s="103" t="str">
+        <x:f>IF(OR(F58="",N58="",N58&lt;=0),"",ROUNDUP(F58/N58,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="37"/>
@@ -4620,13 +4734,15 @@
       <x:c r="K59" s="38"/>
       <x:c r="L59" s="38"/>
       <x:c r="M59" s="38"/>
-      <x:c r="N59" s="38"/>
+      <x:c r="N59" s="50"/>
       <x:c r="O59" s="38"/>
       <x:c r="P59" s="38"/>
       <x:c r="Q59" s="38"/>
       <x:c r="R59" s="38"/>
       <x:c r="S59" s="38"/>
-      <x:c r="T59" s="39"/>
+      <x:c r="T59" s="103" t="str">
+        <x:f>IF(OR(F59="",N59="",N59&lt;=0),"",ROUNDUP(F59/N59,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="37"/>
@@ -4642,13 +4758,15 @@
       <x:c r="K60" s="38"/>
       <x:c r="L60" s="38"/>
       <x:c r="M60" s="38"/>
-      <x:c r="N60" s="38"/>
+      <x:c r="N60" s="50"/>
       <x:c r="O60" s="38"/>
       <x:c r="P60" s="38"/>
       <x:c r="Q60" s="38"/>
       <x:c r="R60" s="38"/>
       <x:c r="S60" s="38"/>
-      <x:c r="T60" s="39"/>
+      <x:c r="T60" s="103" t="str">
+        <x:f>IF(OR(F60="",N60="",N60&lt;=0),"",ROUNDUP(F60/N60,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="37"/>
@@ -4664,13 +4782,15 @@
       <x:c r="K61" s="38"/>
       <x:c r="L61" s="38"/>
       <x:c r="M61" s="38"/>
-      <x:c r="N61" s="38"/>
+      <x:c r="N61" s="50"/>
       <x:c r="O61" s="38"/>
       <x:c r="P61" s="38"/>
       <x:c r="Q61" s="38"/>
       <x:c r="R61" s="38"/>
       <x:c r="S61" s="38"/>
-      <x:c r="T61" s="39"/>
+      <x:c r="T61" s="103" t="str">
+        <x:f>IF(OR(F61="",N61="",N61&lt;=0),"",ROUNDUP(F61/N61,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="37"/>
@@ -4686,13 +4806,15 @@
       <x:c r="K62" s="38"/>
       <x:c r="L62" s="38"/>
       <x:c r="M62" s="38"/>
-      <x:c r="N62" s="38"/>
+      <x:c r="N62" s="50"/>
       <x:c r="O62" s="38"/>
       <x:c r="P62" s="38"/>
       <x:c r="Q62" s="38"/>
       <x:c r="R62" s="38"/>
       <x:c r="S62" s="38"/>
-      <x:c r="T62" s="39"/>
+      <x:c r="T62" s="103" t="str">
+        <x:f>IF(OR(F62="",N62="",N62&lt;=0),"",ROUNDUP(F62/N62,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="37"/>
@@ -4708,13 +4830,15 @@
       <x:c r="K63" s="38"/>
       <x:c r="L63" s="38"/>
       <x:c r="M63" s="38"/>
-      <x:c r="N63" s="38"/>
+      <x:c r="N63" s="50"/>
       <x:c r="O63" s="38"/>
       <x:c r="P63" s="38"/>
       <x:c r="Q63" s="38"/>
       <x:c r="R63" s="38"/>
       <x:c r="S63" s="38"/>
-      <x:c r="T63" s="39"/>
+      <x:c r="T63" s="103" t="str">
+        <x:f>IF(OR(F63="",N63="",N63&lt;=0),"",ROUNDUP(F63/N63,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="37"/>
@@ -4730,13 +4854,15 @@
       <x:c r="K64" s="38"/>
       <x:c r="L64" s="38"/>
       <x:c r="M64" s="38"/>
-      <x:c r="N64" s="38"/>
+      <x:c r="N64" s="50"/>
       <x:c r="O64" s="38"/>
       <x:c r="P64" s="38"/>
       <x:c r="Q64" s="38"/>
       <x:c r="R64" s="38"/>
       <x:c r="S64" s="38"/>
-      <x:c r="T64" s="39"/>
+      <x:c r="T64" s="103" t="str">
+        <x:f>IF(OR(F64="",N64="",N64&lt;=0),"",ROUNDUP(F64/N64,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="37"/>
@@ -4752,13 +4878,15 @@
       <x:c r="K65" s="38"/>
       <x:c r="L65" s="38"/>
       <x:c r="M65" s="38"/>
-      <x:c r="N65" s="38"/>
+      <x:c r="N65" s="50"/>
       <x:c r="O65" s="38"/>
       <x:c r="P65" s="38"/>
       <x:c r="Q65" s="38"/>
       <x:c r="R65" s="38"/>
       <x:c r="S65" s="38"/>
-      <x:c r="T65" s="39"/>
+      <x:c r="T65" s="103" t="str">
+        <x:f>IF(OR(F65="",N65="",N65&lt;=0),"",ROUNDUP(F65/N65,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="37"/>
@@ -4774,13 +4902,15 @@
       <x:c r="K66" s="38"/>
       <x:c r="L66" s="38"/>
       <x:c r="M66" s="38"/>
-      <x:c r="N66" s="38"/>
+      <x:c r="N66" s="50"/>
       <x:c r="O66" s="38"/>
       <x:c r="P66" s="38"/>
       <x:c r="Q66" s="38"/>
       <x:c r="R66" s="38"/>
       <x:c r="S66" s="38"/>
-      <x:c r="T66" s="39"/>
+      <x:c r="T66" s="103" t="str">
+        <x:f>IF(OR(F66="",N66="",N66&lt;=0),"",ROUNDUP(F66/N66,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="37"/>
@@ -4796,13 +4926,15 @@
       <x:c r="K67" s="38"/>
       <x:c r="L67" s="38"/>
       <x:c r="M67" s="38"/>
-      <x:c r="N67" s="38"/>
+      <x:c r="N67" s="50"/>
       <x:c r="O67" s="38"/>
       <x:c r="P67" s="38"/>
       <x:c r="Q67" s="38"/>
       <x:c r="R67" s="38"/>
       <x:c r="S67" s="38"/>
-      <x:c r="T67" s="39"/>
+      <x:c r="T67" s="103" t="str">
+        <x:f>IF(OR(F67="",N67="",N67&lt;=0),"",ROUNDUP(F67/N67,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="37"/>
@@ -4818,13 +4950,15 @@
       <x:c r="K68" s="38"/>
       <x:c r="L68" s="38"/>
       <x:c r="M68" s="38"/>
-      <x:c r="N68" s="38"/>
+      <x:c r="N68" s="50"/>
       <x:c r="O68" s="38"/>
       <x:c r="P68" s="38"/>
       <x:c r="Q68" s="38"/>
       <x:c r="R68" s="38"/>
       <x:c r="S68" s="38"/>
-      <x:c r="T68" s="39"/>
+      <x:c r="T68" s="103" t="str">
+        <x:f>IF(OR(F68="",N68="",N68&lt;=0),"",ROUNDUP(F68/N68,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="37"/>
@@ -4840,13 +4974,15 @@
       <x:c r="K69" s="38"/>
       <x:c r="L69" s="38"/>
       <x:c r="M69" s="38"/>
-      <x:c r="N69" s="38"/>
+      <x:c r="N69" s="50"/>
       <x:c r="O69" s="38"/>
       <x:c r="P69" s="38"/>
       <x:c r="Q69" s="38"/>
       <x:c r="R69" s="38"/>
       <x:c r="S69" s="38"/>
-      <x:c r="T69" s="39"/>
+      <x:c r="T69" s="103" t="str">
+        <x:f>IF(OR(F69="",N69="",N69&lt;=0),"",ROUNDUP(F69/N69,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="37"/>
@@ -4862,13 +4998,15 @@
       <x:c r="K70" s="38"/>
       <x:c r="L70" s="38"/>
       <x:c r="M70" s="38"/>
-      <x:c r="N70" s="38"/>
+      <x:c r="N70" s="50"/>
       <x:c r="O70" s="38"/>
       <x:c r="P70" s="38"/>
       <x:c r="Q70" s="38"/>
       <x:c r="R70" s="38"/>
       <x:c r="S70" s="38"/>
-      <x:c r="T70" s="39"/>
+      <x:c r="T70" s="103" t="str">
+        <x:f>IF(OR(F70="",N70="",N70&lt;=0),"",ROUNDUP(F70/N70,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="37"/>
@@ -4884,13 +5022,15 @@
       <x:c r="K71" s="38"/>
       <x:c r="L71" s="38"/>
       <x:c r="M71" s="38"/>
-      <x:c r="N71" s="38"/>
+      <x:c r="N71" s="50"/>
       <x:c r="O71" s="38"/>
       <x:c r="P71" s="38"/>
       <x:c r="Q71" s="38"/>
       <x:c r="R71" s="38"/>
       <x:c r="S71" s="38"/>
-      <x:c r="T71" s="39"/>
+      <x:c r="T71" s="103" t="str">
+        <x:f>IF(OR(F71="",N71="",N71&lt;=0),"",ROUNDUP(F71/N71,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="37"/>
@@ -4906,13 +5046,15 @@
       <x:c r="K72" s="38"/>
       <x:c r="L72" s="38"/>
       <x:c r="M72" s="38"/>
-      <x:c r="N72" s="38"/>
+      <x:c r="N72" s="50"/>
       <x:c r="O72" s="38"/>
       <x:c r="P72" s="38"/>
       <x:c r="Q72" s="38"/>
       <x:c r="R72" s="38"/>
       <x:c r="S72" s="38"/>
-      <x:c r="T72" s="39"/>
+      <x:c r="T72" s="103" t="str">
+        <x:f>IF(OR(F72="",N72="",N72&lt;=0),"",ROUNDUP(F72/N72,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="37"/>
@@ -4928,13 +5070,15 @@
       <x:c r="K73" s="38"/>
       <x:c r="L73" s="38"/>
       <x:c r="M73" s="38"/>
-      <x:c r="N73" s="38"/>
+      <x:c r="N73" s="50"/>
       <x:c r="O73" s="38"/>
       <x:c r="P73" s="38"/>
       <x:c r="Q73" s="38"/>
       <x:c r="R73" s="38"/>
       <x:c r="S73" s="38"/>
-      <x:c r="T73" s="39"/>
+      <x:c r="T73" s="103" t="str">
+        <x:f>IF(OR(F73="",N73="",N73&lt;=0),"",ROUNDUP(F73/N73,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="37"/>
@@ -4950,13 +5094,15 @@
       <x:c r="K74" s="38"/>
       <x:c r="L74" s="38"/>
       <x:c r="M74" s="38"/>
-      <x:c r="N74" s="38"/>
+      <x:c r="N74" s="50"/>
       <x:c r="O74" s="38"/>
       <x:c r="P74" s="38"/>
       <x:c r="Q74" s="38"/>
       <x:c r="R74" s="38"/>
       <x:c r="S74" s="38"/>
-      <x:c r="T74" s="39"/>
+      <x:c r="T74" s="103" t="str">
+        <x:f>IF(OR(F74="",N74="",N74&lt;=0),"",ROUNDUP(F74/N74,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="37"/>
@@ -4972,13 +5118,15 @@
       <x:c r="K75" s="38"/>
       <x:c r="L75" s="38"/>
       <x:c r="M75" s="38"/>
-      <x:c r="N75" s="38"/>
+      <x:c r="N75" s="50"/>
       <x:c r="O75" s="38"/>
       <x:c r="P75" s="38"/>
       <x:c r="Q75" s="38"/>
       <x:c r="R75" s="38"/>
       <x:c r="S75" s="38"/>
-      <x:c r="T75" s="39"/>
+      <x:c r="T75" s="103" t="str">
+        <x:f>IF(OR(F75="",N75="",N75&lt;=0),"",ROUNDUP(F75/N75,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="37"/>
@@ -4994,13 +5142,15 @@
       <x:c r="K76" s="38"/>
       <x:c r="L76" s="38"/>
       <x:c r="M76" s="38"/>
-      <x:c r="N76" s="38"/>
+      <x:c r="N76" s="50"/>
       <x:c r="O76" s="38"/>
       <x:c r="P76" s="38"/>
       <x:c r="Q76" s="38"/>
       <x:c r="R76" s="38"/>
       <x:c r="S76" s="38"/>
-      <x:c r="T76" s="39"/>
+      <x:c r="T76" s="103" t="str">
+        <x:f>IF(OR(F76="",N76="",N76&lt;=0),"",ROUNDUP(F76/N76,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="37"/>
@@ -5016,13 +5166,15 @@
       <x:c r="K77" s="38"/>
       <x:c r="L77" s="38"/>
       <x:c r="M77" s="38"/>
-      <x:c r="N77" s="38"/>
+      <x:c r="N77" s="50"/>
       <x:c r="O77" s="38"/>
       <x:c r="P77" s="38"/>
       <x:c r="Q77" s="38"/>
       <x:c r="R77" s="38"/>
       <x:c r="S77" s="38"/>
-      <x:c r="T77" s="39"/>
+      <x:c r="T77" s="103" t="str">
+        <x:f>IF(OR(F77="",N77="",N77&lt;=0),"",ROUNDUP(F77/N77,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="37"/>
@@ -5038,13 +5190,15 @@
       <x:c r="K78" s="38"/>
       <x:c r="L78" s="38"/>
       <x:c r="M78" s="38"/>
-      <x:c r="N78" s="38"/>
+      <x:c r="N78" s="50"/>
       <x:c r="O78" s="38"/>
       <x:c r="P78" s="38"/>
       <x:c r="Q78" s="38"/>
       <x:c r="R78" s="38"/>
       <x:c r="S78" s="38"/>
-      <x:c r="T78" s="39"/>
+      <x:c r="T78" s="103" t="str">
+        <x:f>IF(OR(F78="",N78="",N78&lt;=0),"",ROUNDUP(F78/N78,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="37"/>
@@ -5060,13 +5214,15 @@
       <x:c r="K79" s="38"/>
       <x:c r="L79" s="38"/>
       <x:c r="M79" s="38"/>
-      <x:c r="N79" s="38"/>
+      <x:c r="N79" s="50"/>
       <x:c r="O79" s="38"/>
       <x:c r="P79" s="38"/>
       <x:c r="Q79" s="38"/>
       <x:c r="R79" s="38"/>
       <x:c r="S79" s="38"/>
-      <x:c r="T79" s="39"/>
+      <x:c r="T79" s="103" t="str">
+        <x:f>IF(OR(F79="",N79="",N79&lt;=0),"",ROUNDUP(F79/N79,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="37"/>
@@ -5082,13 +5238,15 @@
       <x:c r="K80" s="38"/>
       <x:c r="L80" s="38"/>
       <x:c r="M80" s="38"/>
-      <x:c r="N80" s="38"/>
+      <x:c r="N80" s="50"/>
       <x:c r="O80" s="38"/>
       <x:c r="P80" s="38"/>
       <x:c r="Q80" s="38"/>
       <x:c r="R80" s="38"/>
       <x:c r="S80" s="38"/>
-      <x:c r="T80" s="39"/>
+      <x:c r="T80" s="103" t="str">
+        <x:f>IF(OR(F80="",N80="",N80&lt;=0),"",ROUNDUP(F80/N80,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="37"/>
@@ -5104,13 +5262,15 @@
       <x:c r="K81" s="38"/>
       <x:c r="L81" s="38"/>
       <x:c r="M81" s="38"/>
-      <x:c r="N81" s="38"/>
+      <x:c r="N81" s="50"/>
       <x:c r="O81" s="38"/>
       <x:c r="P81" s="38"/>
       <x:c r="Q81" s="38"/>
       <x:c r="R81" s="38"/>
       <x:c r="S81" s="38"/>
-      <x:c r="T81" s="39"/>
+      <x:c r="T81" s="103" t="str">
+        <x:f>IF(OR(F81="",N81="",N81&lt;=0),"",ROUNDUP(F81/N81,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="37"/>
@@ -5126,13 +5286,15 @@
       <x:c r="K82" s="38"/>
       <x:c r="L82" s="38"/>
       <x:c r="M82" s="38"/>
-      <x:c r="N82" s="38"/>
+      <x:c r="N82" s="50"/>
       <x:c r="O82" s="38"/>
       <x:c r="P82" s="38"/>
       <x:c r="Q82" s="38"/>
       <x:c r="R82" s="38"/>
       <x:c r="S82" s="38"/>
-      <x:c r="T82" s="39"/>
+      <x:c r="T82" s="103" t="str">
+        <x:f>IF(OR(F82="",N82="",N82&lt;=0),"",ROUNDUP(F82/N82,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="37"/>
@@ -5148,13 +5310,15 @@
       <x:c r="K83" s="38"/>
       <x:c r="L83" s="38"/>
       <x:c r="M83" s="38"/>
-      <x:c r="N83" s="38"/>
+      <x:c r="N83" s="50"/>
       <x:c r="O83" s="38"/>
       <x:c r="P83" s="38"/>
       <x:c r="Q83" s="38"/>
       <x:c r="R83" s="38"/>
       <x:c r="S83" s="38"/>
-      <x:c r="T83" s="39"/>
+      <x:c r="T83" s="103" t="str">
+        <x:f>IF(OR(F83="",N83="",N83&lt;=0),"",ROUNDUP(F83/N83,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="37"/>
@@ -5170,13 +5334,15 @@
       <x:c r="K84" s="38"/>
       <x:c r="L84" s="38"/>
       <x:c r="M84" s="38"/>
-      <x:c r="N84" s="38"/>
+      <x:c r="N84" s="50"/>
       <x:c r="O84" s="38"/>
       <x:c r="P84" s="38"/>
       <x:c r="Q84" s="38"/>
       <x:c r="R84" s="38"/>
       <x:c r="S84" s="38"/>
-      <x:c r="T84" s="39"/>
+      <x:c r="T84" s="103" t="str">
+        <x:f>IF(OR(F84="",N84="",N84&lt;=0),"",ROUNDUP(F84/N84,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="37"/>
@@ -5192,13 +5358,15 @@
       <x:c r="K85" s="38"/>
       <x:c r="L85" s="38"/>
       <x:c r="M85" s="38"/>
-      <x:c r="N85" s="38"/>
+      <x:c r="N85" s="50"/>
       <x:c r="O85" s="38"/>
       <x:c r="P85" s="38"/>
       <x:c r="Q85" s="38"/>
       <x:c r="R85" s="38"/>
       <x:c r="S85" s="38"/>
-      <x:c r="T85" s="39"/>
+      <x:c r="T85" s="103" t="str">
+        <x:f>IF(OR(F85="",N85="",N85&lt;=0),"",ROUNDUP(F85/N85,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="37"/>
@@ -5214,13 +5382,15 @@
       <x:c r="K86" s="38"/>
       <x:c r="L86" s="38"/>
       <x:c r="M86" s="38"/>
-      <x:c r="N86" s="38"/>
+      <x:c r="N86" s="50"/>
       <x:c r="O86" s="38"/>
       <x:c r="P86" s="38"/>
       <x:c r="Q86" s="38"/>
       <x:c r="R86" s="38"/>
       <x:c r="S86" s="38"/>
-      <x:c r="T86" s="39"/>
+      <x:c r="T86" s="103" t="str">
+        <x:f>IF(OR(F86="",N86="",N86&lt;=0),"",ROUNDUP(F86/N86,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="37"/>
@@ -5236,13 +5406,15 @@
       <x:c r="K87" s="38"/>
       <x:c r="L87" s="38"/>
       <x:c r="M87" s="38"/>
-      <x:c r="N87" s="38"/>
+      <x:c r="N87" s="50"/>
       <x:c r="O87" s="38"/>
       <x:c r="P87" s="38"/>
       <x:c r="Q87" s="38"/>
       <x:c r="R87" s="38"/>
       <x:c r="S87" s="38"/>
-      <x:c r="T87" s="39"/>
+      <x:c r="T87" s="103" t="str">
+        <x:f>IF(OR(F87="",N87="",N87&lt;=0),"",ROUNDUP(F87/N87,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="37"/>
@@ -5258,13 +5430,15 @@
       <x:c r="K88" s="38"/>
       <x:c r="L88" s="38"/>
       <x:c r="M88" s="38"/>
-      <x:c r="N88" s="38"/>
+      <x:c r="N88" s="50"/>
       <x:c r="O88" s="38"/>
       <x:c r="P88" s="38"/>
       <x:c r="Q88" s="38"/>
       <x:c r="R88" s="38"/>
       <x:c r="S88" s="38"/>
-      <x:c r="T88" s="39"/>
+      <x:c r="T88" s="103" t="str">
+        <x:f>IF(OR(F88="",N88="",N88&lt;=0),"",ROUNDUP(F88/N88,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="37"/>
@@ -5280,13 +5454,15 @@
       <x:c r="K89" s="38"/>
       <x:c r="L89" s="38"/>
       <x:c r="M89" s="38"/>
-      <x:c r="N89" s="38"/>
+      <x:c r="N89" s="50"/>
       <x:c r="O89" s="38"/>
       <x:c r="P89" s="38"/>
       <x:c r="Q89" s="38"/>
       <x:c r="R89" s="38"/>
       <x:c r="S89" s="38"/>
-      <x:c r="T89" s="39"/>
+      <x:c r="T89" s="103" t="str">
+        <x:f>IF(OR(F89="",N89="",N89&lt;=0),"",ROUNDUP(F89/N89,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="37"/>
@@ -5302,13 +5478,15 @@
       <x:c r="K90" s="38"/>
       <x:c r="L90" s="38"/>
       <x:c r="M90" s="38"/>
-      <x:c r="N90" s="38"/>
+      <x:c r="N90" s="50"/>
       <x:c r="O90" s="38"/>
       <x:c r="P90" s="38"/>
       <x:c r="Q90" s="38"/>
       <x:c r="R90" s="38"/>
       <x:c r="S90" s="38"/>
-      <x:c r="T90" s="39"/>
+      <x:c r="T90" s="103" t="str">
+        <x:f>IF(OR(F90="",N90="",N90&lt;=0),"",ROUNDUP(F90/N90,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="37"/>
@@ -5324,13 +5502,15 @@
       <x:c r="K91" s="38"/>
       <x:c r="L91" s="38"/>
       <x:c r="M91" s="38"/>
-      <x:c r="N91" s="38"/>
+      <x:c r="N91" s="50"/>
       <x:c r="O91" s="38"/>
       <x:c r="P91" s="38"/>
       <x:c r="Q91" s="38"/>
       <x:c r="R91" s="38"/>
       <x:c r="S91" s="38"/>
-      <x:c r="T91" s="39"/>
+      <x:c r="T91" s="103" t="str">
+        <x:f>IF(OR(F91="",N91="",N91&lt;=0),"",ROUNDUP(F91/N91,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="37"/>
@@ -5346,13 +5526,15 @@
       <x:c r="K92" s="38"/>
       <x:c r="L92" s="38"/>
       <x:c r="M92" s="38"/>
-      <x:c r="N92" s="38"/>
+      <x:c r="N92" s="50"/>
       <x:c r="O92" s="38"/>
       <x:c r="P92" s="38"/>
       <x:c r="Q92" s="38"/>
       <x:c r="R92" s="38"/>
       <x:c r="S92" s="38"/>
-      <x:c r="T92" s="39"/>
+      <x:c r="T92" s="103" t="str">
+        <x:f>IF(OR(F92="",N92="",N92&lt;=0),"",ROUNDUP(F92/N92,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="37"/>
@@ -5368,13 +5550,15 @@
       <x:c r="K93" s="38"/>
       <x:c r="L93" s="38"/>
       <x:c r="M93" s="38"/>
-      <x:c r="N93" s="38"/>
+      <x:c r="N93" s="50"/>
       <x:c r="O93" s="38"/>
       <x:c r="P93" s="38"/>
       <x:c r="Q93" s="38"/>
       <x:c r="R93" s="38"/>
       <x:c r="S93" s="38"/>
-      <x:c r="T93" s="39"/>
+      <x:c r="T93" s="103" t="str">
+        <x:f>IF(OR(F93="",N93="",N93&lt;=0),"",ROUNDUP(F93/N93,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="37"/>
@@ -5390,13 +5574,15 @@
       <x:c r="K94" s="38"/>
       <x:c r="L94" s="38"/>
       <x:c r="M94" s="38"/>
-      <x:c r="N94" s="38"/>
+      <x:c r="N94" s="50"/>
       <x:c r="O94" s="38"/>
       <x:c r="P94" s="38"/>
       <x:c r="Q94" s="38"/>
       <x:c r="R94" s="38"/>
       <x:c r="S94" s="38"/>
-      <x:c r="T94" s="39"/>
+      <x:c r="T94" s="103" t="str">
+        <x:f>IF(OR(F94="",N94="",N94&lt;=0),"",ROUNDUP(F94/N94,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="37"/>
@@ -5412,13 +5598,15 @@
       <x:c r="K95" s="38"/>
       <x:c r="L95" s="38"/>
       <x:c r="M95" s="38"/>
-      <x:c r="N95" s="38"/>
+      <x:c r="N95" s="50"/>
       <x:c r="O95" s="38"/>
       <x:c r="P95" s="38"/>
       <x:c r="Q95" s="38"/>
       <x:c r="R95" s="38"/>
       <x:c r="S95" s="38"/>
-      <x:c r="T95" s="39"/>
+      <x:c r="T95" s="103" t="str">
+        <x:f>IF(OR(F95="",N95="",N95&lt;=0),"",ROUNDUP(F95/N95,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="37"/>
@@ -5434,13 +5622,15 @@
       <x:c r="K96" s="38"/>
       <x:c r="L96" s="38"/>
       <x:c r="M96" s="38"/>
-      <x:c r="N96" s="38"/>
+      <x:c r="N96" s="50"/>
       <x:c r="O96" s="38"/>
       <x:c r="P96" s="38"/>
       <x:c r="Q96" s="38"/>
       <x:c r="R96" s="38"/>
       <x:c r="S96" s="38"/>
-      <x:c r="T96" s="39"/>
+      <x:c r="T96" s="103" t="str">
+        <x:f>IF(OR(F96="",N96="",N96&lt;=0),"",ROUNDUP(F96/N96,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="37"/>
@@ -5456,13 +5646,15 @@
       <x:c r="K97" s="38"/>
       <x:c r="L97" s="38"/>
       <x:c r="M97" s="38"/>
-      <x:c r="N97" s="38"/>
+      <x:c r="N97" s="50"/>
       <x:c r="O97" s="38"/>
       <x:c r="P97" s="38"/>
       <x:c r="Q97" s="38"/>
       <x:c r="R97" s="38"/>
       <x:c r="S97" s="38"/>
-      <x:c r="T97" s="39"/>
+      <x:c r="T97" s="103" t="str">
+        <x:f>IF(OR(F97="",N97="",N97&lt;=0),"",ROUNDUP(F97/N97,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="37"/>
@@ -5478,13 +5670,15 @@
       <x:c r="K98" s="38"/>
       <x:c r="L98" s="38"/>
       <x:c r="M98" s="38"/>
-      <x:c r="N98" s="38"/>
+      <x:c r="N98" s="50"/>
       <x:c r="O98" s="38"/>
       <x:c r="P98" s="38"/>
       <x:c r="Q98" s="38"/>
       <x:c r="R98" s="38"/>
       <x:c r="S98" s="38"/>
-      <x:c r="T98" s="39"/>
+      <x:c r="T98" s="103" t="str">
+        <x:f>IF(OR(F98="",N98="",N98&lt;=0),"",ROUNDUP(F98/N98,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="37"/>
@@ -5500,13 +5694,15 @@
       <x:c r="K99" s="38"/>
       <x:c r="L99" s="38"/>
       <x:c r="M99" s="38"/>
-      <x:c r="N99" s="38"/>
+      <x:c r="N99" s="50"/>
       <x:c r="O99" s="38"/>
       <x:c r="P99" s="38"/>
       <x:c r="Q99" s="38"/>
       <x:c r="R99" s="38"/>
       <x:c r="S99" s="38"/>
-      <x:c r="T99" s="39"/>
+      <x:c r="T99" s="103" t="str">
+        <x:f>IF(OR(F99="",N99="",N99&lt;=0),"",ROUNDUP(F99/N99,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="37"/>
@@ -5522,13 +5718,15 @@
       <x:c r="K100" s="38"/>
       <x:c r="L100" s="38"/>
       <x:c r="M100" s="38"/>
-      <x:c r="N100" s="38"/>
+      <x:c r="N100" s="50"/>
       <x:c r="O100" s="38"/>
       <x:c r="P100" s="38"/>
       <x:c r="Q100" s="38"/>
       <x:c r="R100" s="38"/>
       <x:c r="S100" s="38"/>
-      <x:c r="T100" s="39"/>
+      <x:c r="T100" s="103" t="str">
+        <x:f>IF(OR(F100="",N100="",N100&lt;=0),"",ROUNDUP(F100/N100,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="37"/>
@@ -5544,13 +5742,15 @@
       <x:c r="K101" s="38"/>
       <x:c r="L101" s="38"/>
       <x:c r="M101" s="38"/>
-      <x:c r="N101" s="38"/>
+      <x:c r="N101" s="50"/>
       <x:c r="O101" s="38"/>
       <x:c r="P101" s="38"/>
       <x:c r="Q101" s="38"/>
       <x:c r="R101" s="38"/>
       <x:c r="S101" s="38"/>
-      <x:c r="T101" s="39"/>
+      <x:c r="T101" s="103" t="str">
+        <x:f>IF(OR(F101="",N101="",N101&lt;=0),"",ROUNDUP(F101/N101,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="37"/>
@@ -5566,13 +5766,15 @@
       <x:c r="K102" s="38"/>
       <x:c r="L102" s="38"/>
       <x:c r="M102" s="38"/>
-      <x:c r="N102" s="38"/>
+      <x:c r="N102" s="50"/>
       <x:c r="O102" s="38"/>
       <x:c r="P102" s="38"/>
       <x:c r="Q102" s="38"/>
       <x:c r="R102" s="38"/>
       <x:c r="S102" s="38"/>
-      <x:c r="T102" s="39"/>
+      <x:c r="T102" s="103" t="str">
+        <x:f>IF(OR(F102="",N102="",N102&lt;=0),"",ROUNDUP(F102/N102,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="37"/>
@@ -5588,13 +5790,15 @@
       <x:c r="K103" s="38"/>
       <x:c r="L103" s="38"/>
       <x:c r="M103" s="38"/>
-      <x:c r="N103" s="38"/>
+      <x:c r="N103" s="50"/>
       <x:c r="O103" s="38"/>
       <x:c r="P103" s="38"/>
       <x:c r="Q103" s="38"/>
       <x:c r="R103" s="38"/>
       <x:c r="S103" s="38"/>
-      <x:c r="T103" s="39"/>
+      <x:c r="T103" s="103" t="str">
+        <x:f>IF(OR(F103="",N103="",N103&lt;=0),"",ROUNDUP(F103/N103,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="37"/>
@@ -5610,13 +5814,15 @@
       <x:c r="K104" s="38"/>
       <x:c r="L104" s="38"/>
       <x:c r="M104" s="38"/>
-      <x:c r="N104" s="38"/>
+      <x:c r="N104" s="50"/>
       <x:c r="O104" s="38"/>
       <x:c r="P104" s="38"/>
       <x:c r="Q104" s="38"/>
       <x:c r="R104" s="38"/>
       <x:c r="S104" s="38"/>
-      <x:c r="T104" s="39"/>
+      <x:c r="T104" s="103" t="str">
+        <x:f>IF(OR(F104="",N104="",N104&lt;=0),"",ROUNDUP(F104/N104,0))</x:f>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="40"/>
@@ -5632,13 +5838,15 @@
       <x:c r="K105" s="41"/>
       <x:c r="L105" s="41"/>
       <x:c r="M105" s="41"/>
-      <x:c r="N105" s="41"/>
+      <x:c r="N105" s="51"/>
       <x:c r="O105" s="41"/>
       <x:c r="P105" s="41"/>
       <x:c r="Q105" s="41"/>
       <x:c r="R105" s="41"/>
       <x:c r="S105" s="41"/>
-      <x:c r="T105" s="42"/>
+      <x:c r="T105" s="104" t="str">
+        <x:f>IF(OR(F105="",N105="",N105&lt;=0),"",ROUNDUP(F105/N105,0))</x:f>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5906,7 +6114,7 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="84" t="str">
-        <x:v>单件用量</x:v>
+        <x:v>每箱个数</x:v>
       </x:c>
       <x:c r="B17" s="97" t="str">
         <x:v>是</x:v>
@@ -5915,10 +6123,10 @@
         <x:v>usage_quantity</x:v>
       </x:c>
       <x:c r="D17" s="85" t="n">
-        <x:v>0.008333333333333333</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="E17" s="86" t="str">
-        <x:v>必须大于 0；需求数量自动计算。</x:v>
+        <x:v>必须大于 0；纸箱数量按“产品订单数量 ÷ 每箱个数”计算，不足一箱向上取整。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -6008,7 +6216,7 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="87" t="str">
-        <x:v>需求数量</x:v>
+        <x:v>纸箱数量（自动校验）</x:v>
       </x:c>
       <x:c r="B23" s="98" t="str">
         <x:v>系统计算</x:v>
@@ -6020,7 +6228,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="E23" s="89" t="str">
-        <x:v>产品订单数量 × 单件用量，不参与导入。</x:v>
+        <x:v>产品订单数量 ÷ 每箱个数并向上取整；模板公式列，不参与导入。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: add scoped spreadsheet merge and carton templates
</commit_message>
<xml_diff>
--- a/public/templates/carton-history-order-import-template.xlsx
+++ b/public/templates/carton-history-order-import-template.xlsx
@@ -778,6 +778,7 @@
     <col min="31" max="31" width="17" hidden="0" customWidth="1"/>
     <col min="33" max="33" width="24" hidden="0" customWidth="1"/>
     <col min="32" max="32" width="12" hidden="0" customWidth="1"/>
+    <col min="34" max="34" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -830,6 +831,11 @@
         <v>选填</v>
       </c>
       <c r="AG1" s="51"/>
+      <c r="AH1" s="51" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="6" t="str">
@@ -930,6 +936,11 @@
       </c>
       <c r="AG2" s="12" t="str">
         <v>历史订单号</v>
+      </c>
+      <c r="AH2" s="12" t="inlineStr">
+        <is>
+          <t>客户PO</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
@@ -966,6 +977,7 @@
       <c r="AE3" s="48"/>
       <c r="AF3" s="21"/>
       <c r="AG3" s="21"/>
+      <c r="AH3" s="21"/>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="19"/>
@@ -1001,6 +1013,7 @@
       <c r="AE4" s="49"/>
       <c r="AF4" s="22"/>
       <c r="AG4" s="22"/>
+      <c r="AH4" s="22"/>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="19"/>
@@ -1036,6 +1049,7 @@
       <c r="AE5" s="49"/>
       <c r="AF5" s="22"/>
       <c r="AG5" s="22"/>
+      <c r="AH5" s="22"/>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="19"/>
@@ -1071,6 +1085,7 @@
       <c r="AE6" s="49"/>
       <c r="AF6" s="22"/>
       <c r="AG6" s="22"/>
+      <c r="AH6" s="22"/>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="19"/>
@@ -1106,6 +1121,7 @@
       <c r="AE7" s="49"/>
       <c r="AF7" s="22"/>
       <c r="AG7" s="22"/>
+      <c r="AH7" s="22"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19"/>
@@ -1141,6 +1157,7 @@
       <c r="AE8" s="49"/>
       <c r="AF8" s="22"/>
       <c r="AG8" s="22"/>
+      <c r="AH8" s="22"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="19"/>
@@ -1176,6 +1193,7 @@
       <c r="AE9" s="49"/>
       <c r="AF9" s="22"/>
       <c r="AG9" s="22"/>
+      <c r="AH9" s="22"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="19"/>
@@ -1211,6 +1229,7 @@
       <c r="AE10" s="49"/>
       <c r="AF10" s="22"/>
       <c r="AG10" s="22"/>
+      <c r="AH10" s="22"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="19"/>
@@ -1246,6 +1265,7 @@
       <c r="AE11" s="49"/>
       <c r="AF11" s="22"/>
       <c r="AG11" s="22"/>
+      <c r="AH11" s="22"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="19"/>
@@ -1281,6 +1301,7 @@
       <c r="AE12" s="49"/>
       <c r="AF12" s="22"/>
       <c r="AG12" s="22"/>
+      <c r="AH12" s="22"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="19"/>
@@ -1316,6 +1337,7 @@
       <c r="AE13" s="49"/>
       <c r="AF13" s="22"/>
       <c r="AG13" s="22"/>
+      <c r="AH13" s="22"/>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="19"/>
@@ -1351,6 +1373,7 @@
       <c r="AE14" s="49"/>
       <c r="AF14" s="22"/>
       <c r="AG14" s="22"/>
+      <c r="AH14" s="22"/>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="19"/>
@@ -1386,6 +1409,7 @@
       <c r="AE15" s="49"/>
       <c r="AF15" s="22"/>
       <c r="AG15" s="22"/>
+      <c r="AH15" s="22"/>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="19"/>
@@ -1421,6 +1445,7 @@
       <c r="AE16" s="49"/>
       <c r="AF16" s="22"/>
       <c r="AG16" s="22"/>
+      <c r="AH16" s="22"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="19"/>
@@ -1456,6 +1481,7 @@
       <c r="AE17" s="49"/>
       <c r="AF17" s="22"/>
       <c r="AG17" s="22"/>
+      <c r="AH17" s="22"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="19"/>
@@ -1491,6 +1517,7 @@
       <c r="AE18" s="49"/>
       <c r="AF18" s="22"/>
       <c r="AG18" s="22"/>
+      <c r="AH18" s="22"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="19"/>
@@ -1526,6 +1553,7 @@
       <c r="AE19" s="49"/>
       <c r="AF19" s="22"/>
       <c r="AG19" s="22"/>
+      <c r="AH19" s="22"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="19"/>
@@ -1561,6 +1589,7 @@
       <c r="AE20" s="49"/>
       <c r="AF20" s="22"/>
       <c r="AG20" s="22"/>
+      <c r="AH20" s="22"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="19"/>
@@ -1596,6 +1625,7 @@
       <c r="AE21" s="49"/>
       <c r="AF21" s="22"/>
       <c r="AG21" s="22"/>
+      <c r="AH21" s="22"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="19"/>
@@ -1631,6 +1661,7 @@
       <c r="AE22" s="49"/>
       <c r="AF22" s="22"/>
       <c r="AG22" s="22"/>
+      <c r="AH22" s="22"/>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="19"/>
@@ -1666,6 +1697,7 @@
       <c r="AE23" s="49"/>
       <c r="AF23" s="22"/>
       <c r="AG23" s="22"/>
+      <c r="AH23" s="22"/>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="19"/>
@@ -1701,6 +1733,7 @@
       <c r="AE24" s="49"/>
       <c r="AF24" s="22"/>
       <c r="AG24" s="22"/>
+      <c r="AH24" s="22"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="19"/>
@@ -1736,6 +1769,7 @@
       <c r="AE25" s="49"/>
       <c r="AF25" s="22"/>
       <c r="AG25" s="22"/>
+      <c r="AH25" s="22"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="19"/>
@@ -1771,6 +1805,7 @@
       <c r="AE26" s="49"/>
       <c r="AF26" s="22"/>
       <c r="AG26" s="22"/>
+      <c r="AH26" s="22"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="19"/>
@@ -1806,6 +1841,7 @@
       <c r="AE27" s="49"/>
       <c r="AF27" s="22"/>
       <c r="AG27" s="22"/>
+      <c r="AH27" s="22"/>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="19"/>
@@ -1841,6 +1877,7 @@
       <c r="AE28" s="49"/>
       <c r="AF28" s="22"/>
       <c r="AG28" s="22"/>
+      <c r="AH28" s="22"/>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="19"/>
@@ -1876,6 +1913,7 @@
       <c r="AE29" s="49"/>
       <c r="AF29" s="22"/>
       <c r="AG29" s="22"/>
+      <c r="AH29" s="22"/>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="19"/>
@@ -1911,6 +1949,7 @@
       <c r="AE30" s="49"/>
       <c r="AF30" s="22"/>
       <c r="AG30" s="22"/>
+      <c r="AH30" s="22"/>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="19"/>
@@ -1946,6 +1985,7 @@
       <c r="AE31" s="49"/>
       <c r="AF31" s="22"/>
       <c r="AG31" s="22"/>
+      <c r="AH31" s="22"/>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="20"/>
@@ -1981,6 +2021,7 @@
       <c r="AE32" s="50"/>
       <c r="AF32" s="23"/>
       <c r="AG32" s="23"/>
+      <c r="AH32" s="23"/>
     </row>
   </sheetData>
   <dataValidations count="7">
@@ -2601,6 +2642,7 @@
     <x:col min="31" max="31" width="17" hidden="0" customWidth="1"/>
     <x:col min="33" max="33" width="24" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="12" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="22" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2851,6 +2893,11 @@
       <x:c r="AG5" s="12" t="str">
         <x:v>历史订单号</x:v>
       </x:c>
+      <x:c r="AH5" s="12" t="inlineStr">
+        <x:is>
+          <x:t>客户PO</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="21" t="str">
@@ -3237,8 +3284,16 @@
       <x:c r="H14" s="6" t="str">
         <x:v>每箱个数</x:v>
       </x:c>
-      <x:c r="I14" s="83"/>
-      <x:c r="J14" s="83"/>
+      <x:c r="I14" s="83" t="inlineStr">
+        <x:is>
+          <x:t>每箱净重kg</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J14" s="83" t="inlineStr">
+        <x:is>
+          <x:t>每箱毛重kg</x:t>
+        </x:is>
+      </x:c>
       <x:c r="K14" s="6" t="str">
         <x:v>单价</x:v>
       </x:c>
@@ -3582,11 +3637,15 @@
       <x:c r="A16" s="72" t="str">
         <x:v>客户交期（选填）</x:v>
       </x:c>
-      <x:c r="B16" s="69" t="str">
-        <x:v>有客户交期才填写完整日期。</x:v>
-      </x:c>
-      <x:c r="C16" s="69" t="str">
-        <x:v>与计划交期分别保留，不擅自补成同一天。</x:v>
+      <x:c r="B16" s="69" t="inlineStr">
+        <x:is>
+          <x:t>有客户交期时填写完整日期；未知可留空。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="69" t="inlineStr">
+        <x:is>
+          <x:t>保留原计划交期；缺客户交期时按计划交期加有效采购安全天数补齐，预览显示实际规则。</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -3677,10 +3736,22 @@
         <x:v>毛重不能小于净重，最多 4 位小数；其他纸品的独立重量可填附加纸品明细。</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="28" customHeight="1">
-      <x:c r="A25" s="2"/>
-      <x:c r="B25" s="2"/>
-      <x:c r="C25" s="2"/>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="72" t="inlineStr">
+        <x:is>
+          <x:t>客户PO（选填）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="69" t="inlineStr">
+        <x:is>
+          <x:t>按原表填写，设置为文本并保留前导0。同客户、合同、货号下不同客户PO须分别填写。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="69" t="inlineStr">
+        <x:is>
+          <x:t>空白保留旧资料兼容；不同非空客户PO用于区分订单，不以合同号替填。</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="2"/>

</xml_diff>

<commit_message>
feat: integrate carton, warehouse and business workspace updates
</commit_message>
<xml_diff>
--- a/public/templates/carton-history-order-import-template.xlsx
+++ b/public/templates/carton-history-order-import-template.xlsx
@@ -778,6 +778,7 @@
     <col min="31" max="31" width="17" hidden="0" customWidth="1"/>
     <col min="33" max="33" width="24" hidden="0" customWidth="1"/>
     <col min="32" max="32" width="12" hidden="0" customWidth="1"/>
+    <col min="34" max="34" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -830,6 +831,11 @@
         <v>选填</v>
       </c>
       <c r="AG1" s="51"/>
+      <c r="AH1" s="51" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="6" t="str">
@@ -930,6 +936,11 @@
       </c>
       <c r="AG2" s="12" t="str">
         <v>历史订单号</v>
+      </c>
+      <c r="AH2" s="12" t="inlineStr">
+        <is>
+          <t>客户PO</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
@@ -966,6 +977,7 @@
       <c r="AE3" s="48"/>
       <c r="AF3" s="21"/>
       <c r="AG3" s="21"/>
+      <c r="AH3" s="21"/>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="19"/>
@@ -1001,6 +1013,7 @@
       <c r="AE4" s="49"/>
       <c r="AF4" s="22"/>
       <c r="AG4" s="22"/>
+      <c r="AH4" s="22"/>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="19"/>
@@ -1036,6 +1049,7 @@
       <c r="AE5" s="49"/>
       <c r="AF5" s="22"/>
       <c r="AG5" s="22"/>
+      <c r="AH5" s="22"/>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="19"/>
@@ -1071,6 +1085,7 @@
       <c r="AE6" s="49"/>
       <c r="AF6" s="22"/>
       <c r="AG6" s="22"/>
+      <c r="AH6" s="22"/>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="19"/>
@@ -1106,6 +1121,7 @@
       <c r="AE7" s="49"/>
       <c r="AF7" s="22"/>
       <c r="AG7" s="22"/>
+      <c r="AH7" s="22"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19"/>
@@ -1141,6 +1157,7 @@
       <c r="AE8" s="49"/>
       <c r="AF8" s="22"/>
       <c r="AG8" s="22"/>
+      <c r="AH8" s="22"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="19"/>
@@ -1176,6 +1193,7 @@
       <c r="AE9" s="49"/>
       <c r="AF9" s="22"/>
       <c r="AG9" s="22"/>
+      <c r="AH9" s="22"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="19"/>
@@ -1211,6 +1229,7 @@
       <c r="AE10" s="49"/>
       <c r="AF10" s="22"/>
       <c r="AG10" s="22"/>
+      <c r="AH10" s="22"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="19"/>
@@ -1246,6 +1265,7 @@
       <c r="AE11" s="49"/>
       <c r="AF11" s="22"/>
       <c r="AG11" s="22"/>
+      <c r="AH11" s="22"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="19"/>
@@ -1281,6 +1301,7 @@
       <c r="AE12" s="49"/>
       <c r="AF12" s="22"/>
       <c r="AG12" s="22"/>
+      <c r="AH12" s="22"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="19"/>
@@ -1316,6 +1337,7 @@
       <c r="AE13" s="49"/>
       <c r="AF13" s="22"/>
       <c r="AG13" s="22"/>
+      <c r="AH13" s="22"/>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="19"/>
@@ -1351,6 +1373,7 @@
       <c r="AE14" s="49"/>
       <c r="AF14" s="22"/>
       <c r="AG14" s="22"/>
+      <c r="AH14" s="22"/>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="19"/>
@@ -1386,6 +1409,7 @@
       <c r="AE15" s="49"/>
       <c r="AF15" s="22"/>
       <c r="AG15" s="22"/>
+      <c r="AH15" s="22"/>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="19"/>
@@ -1421,6 +1445,7 @@
       <c r="AE16" s="49"/>
       <c r="AF16" s="22"/>
       <c r="AG16" s="22"/>
+      <c r="AH16" s="22"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="19"/>
@@ -1456,6 +1481,7 @@
       <c r="AE17" s="49"/>
       <c r="AF17" s="22"/>
       <c r="AG17" s="22"/>
+      <c r="AH17" s="22"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="19"/>
@@ -1491,6 +1517,7 @@
       <c r="AE18" s="49"/>
       <c r="AF18" s="22"/>
       <c r="AG18" s="22"/>
+      <c r="AH18" s="22"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="19"/>
@@ -1526,6 +1553,7 @@
       <c r="AE19" s="49"/>
       <c r="AF19" s="22"/>
       <c r="AG19" s="22"/>
+      <c r="AH19" s="22"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="19"/>
@@ -1561,6 +1589,7 @@
       <c r="AE20" s="49"/>
       <c r="AF20" s="22"/>
       <c r="AG20" s="22"/>
+      <c r="AH20" s="22"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="19"/>
@@ -1596,6 +1625,7 @@
       <c r="AE21" s="49"/>
       <c r="AF21" s="22"/>
       <c r="AG21" s="22"/>
+      <c r="AH21" s="22"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="19"/>
@@ -1631,6 +1661,7 @@
       <c r="AE22" s="49"/>
       <c r="AF22" s="22"/>
       <c r="AG22" s="22"/>
+      <c r="AH22" s="22"/>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="19"/>
@@ -1666,6 +1697,7 @@
       <c r="AE23" s="49"/>
       <c r="AF23" s="22"/>
       <c r="AG23" s="22"/>
+      <c r="AH23" s="22"/>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="19"/>
@@ -1701,6 +1733,7 @@
       <c r="AE24" s="49"/>
       <c r="AF24" s="22"/>
       <c r="AG24" s="22"/>
+      <c r="AH24" s="22"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="19"/>
@@ -1736,6 +1769,7 @@
       <c r="AE25" s="49"/>
       <c r="AF25" s="22"/>
       <c r="AG25" s="22"/>
+      <c r="AH25" s="22"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="19"/>
@@ -1771,6 +1805,7 @@
       <c r="AE26" s="49"/>
       <c r="AF26" s="22"/>
       <c r="AG26" s="22"/>
+      <c r="AH26" s="22"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="19"/>
@@ -1806,6 +1841,7 @@
       <c r="AE27" s="49"/>
       <c r="AF27" s="22"/>
       <c r="AG27" s="22"/>
+      <c r="AH27" s="22"/>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="19"/>
@@ -1841,6 +1877,7 @@
       <c r="AE28" s="49"/>
       <c r="AF28" s="22"/>
       <c r="AG28" s="22"/>
+      <c r="AH28" s="22"/>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="19"/>
@@ -1876,6 +1913,7 @@
       <c r="AE29" s="49"/>
       <c r="AF29" s="22"/>
       <c r="AG29" s="22"/>
+      <c r="AH29" s="22"/>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="19"/>
@@ -1911,6 +1949,7 @@
       <c r="AE30" s="49"/>
       <c r="AF30" s="22"/>
       <c r="AG30" s="22"/>
+      <c r="AH30" s="22"/>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="19"/>
@@ -1946,6 +1985,7 @@
       <c r="AE31" s="49"/>
       <c r="AF31" s="22"/>
       <c r="AG31" s="22"/>
+      <c r="AH31" s="22"/>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="20"/>
@@ -1981,6 +2021,7 @@
       <c r="AE32" s="50"/>
       <c r="AF32" s="23"/>
       <c r="AG32" s="23"/>
+      <c r="AH32" s="23"/>
     </row>
   </sheetData>
   <dataValidations count="7">
@@ -2601,6 +2642,7 @@
     <x:col min="31" max="31" width="17" hidden="0" customWidth="1"/>
     <x:col min="33" max="33" width="24" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="12" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="22" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2851,6 +2893,11 @@
       <x:c r="AG5" s="12" t="str">
         <x:v>历史订单号</x:v>
       </x:c>
+      <x:c r="AH5" s="12" t="inlineStr">
+        <x:is>
+          <x:t>客户PO</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="21" t="str">
@@ -3237,8 +3284,16 @@
       <x:c r="H14" s="6" t="str">
         <x:v>每箱个数</x:v>
       </x:c>
-      <x:c r="I14" s="83"/>
-      <x:c r="J14" s="83"/>
+      <x:c r="I14" s="83" t="inlineStr">
+        <x:is>
+          <x:t>每箱净重kg</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J14" s="83" t="inlineStr">
+        <x:is>
+          <x:t>每箱毛重kg</x:t>
+        </x:is>
+      </x:c>
       <x:c r="K14" s="6" t="str">
         <x:v>单价</x:v>
       </x:c>
@@ -3582,11 +3637,15 @@
       <x:c r="A16" s="72" t="str">
         <x:v>客户交期（选填）</x:v>
       </x:c>
-      <x:c r="B16" s="69" t="str">
-        <x:v>有客户交期才填写完整日期。</x:v>
-      </x:c>
-      <x:c r="C16" s="69" t="str">
-        <x:v>与计划交期分别保留，不擅自补成同一天。</x:v>
+      <x:c r="B16" s="69" t="inlineStr">
+        <x:is>
+          <x:t>有客户交期时填写完整日期；未知可留空。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="69" t="inlineStr">
+        <x:is>
+          <x:t>保留原计划交期；缺客户交期时按计划交期加有效采购安全天数补齐，预览显示实际规则。</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -3677,10 +3736,22 @@
         <x:v>毛重不能小于净重，最多 4 位小数；其他纸品的独立重量可填附加纸品明细。</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="28" customHeight="1">
-      <x:c r="A25" s="2"/>
-      <x:c r="B25" s="2"/>
-      <x:c r="C25" s="2"/>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="72" t="inlineStr">
+        <x:is>
+          <x:t>客户PO（选填）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="69" t="inlineStr">
+        <x:is>
+          <x:t>按原表填写，设置为文本并保留前导0。同客户、合同、货号下不同客户PO须分别填写。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="69" t="inlineStr">
+        <x:is>
+          <x:t>空白保留旧资料兼容；不同非空客户PO用于区分订单，不以合同号替填。</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="2"/>

</xml_diff>